<commit_message>
Add journal/calculator tabs, watchlist scanner, and twice-daily auto-refresh
- Excel: new Journal tab (formula-computed P&L and R-multiples) and
  Calc — Sizing & RR tab (interactive position sizing, 25-50-25 pyramid
  split, weighted R:R, payoff ratio, break-even win rate)
- Father: COLPAL fully exited (600 units, ~-2.5L realized), GILLETTE
  re-tagged HOLD_FOR_TLH pending tax-loss harvesting plan
- watchlist_scan.py: checks structured zones/invalidations per ticker,
  regime gauges vs 21D EMA, --market IN/US filter, markdown report
- GitHub Actions workflow: refreshes tracker + scan at 08:40 IST (IN)
  and 19:40 IST (US) on weekdays, pushes results to branch

https://claude.ai/code/session_01HhF36NsLiVFyxhhXe4S24m
</commit_message>
<xml_diff>
--- a/examples/swing_monitor/Portfolio_Tracker.xlsx
+++ b/examples/swing_monitor/Portfolio_Tracker.xlsx
@@ -13,7 +13,9 @@
     <sheet name="Mutual Funds" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="US Holdings" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Swing &amp; Watchlist" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Father" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Journal" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Calc — Sizing &amp; RR" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Father" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,12 +24,15 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="+0.00;-0.00"/>
     <numFmt numFmtId="165" formatCode="+0.0;-0.0"/>
     <numFmt numFmtId="166" formatCode="0.000"/>
+    <numFmt numFmtId="167" formatCode="+0.0%;-0.0%"/>
+    <numFmt numFmtId="168" formatCode="0.0"/>
+    <numFmt numFmtId="169" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -63,6 +68,17 @@
     </font>
     <font>
       <b val="1"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
       <sz val="9"/>
     </font>
     <font>
@@ -70,7 +86,7 @@
       <sz val="16"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -89,12 +105,22 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00FEF9C3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F0F9FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00DCFCE7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FEE2E2"/>
+        <fgColor rgb="00FEF3C7"/>
       </patternFill>
     </fill>
     <fill>
@@ -120,9 +146,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -148,9 +174,23 @@
     <xf numFmtId="3" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -535,7 +575,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-12 10:37  |  USD/INR 95.0  |  prices: override file (2026-08-12T10:29:00+00:00), yfinance off</t>
+          <t>Generated 2026-08-12 10:58  |  USD/INR 95.0  |  prices: override file (2026-08-12T10:29:00+00:00), yfinance off</t>
         </is>
       </c>
     </row>
@@ -674,7 +714,7 @@
         </is>
       </c>
       <c r="B14" s="11" t="n">
-        <v>7562450</v>
+        <v>6356450</v>
       </c>
     </row>
     <row r="15">
@@ -684,7 +724,7 @@
         </is>
       </c>
       <c r="B15" s="11" t="n">
-        <v>8350431</v>
+        <v>6893503</v>
       </c>
     </row>
     <row r="16">
@@ -694,7 +734,7 @@
         </is>
       </c>
       <c r="B16" s="12" t="n">
-        <v>-787981</v>
+        <v>-537053</v>
       </c>
     </row>
   </sheetData>
@@ -3872,6 +3912,1050 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:L19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="5" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>SWING TRADE JOURNAL — add new rows below; P&amp;L / R computed by formula</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>Cur</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>Date In</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>Date Out</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>Avg Entry</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>Avg Exit</t>
+        </is>
+      </c>
+      <c r="I2" s="4" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="J2" s="4" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+      <c r="K2" s="4" t="inlineStr">
+        <is>
+          <t>P&amp;L %</t>
+        </is>
+      </c>
+      <c r="L2" s="4" t="inlineStr">
+        <is>
+          <t>R-multiple</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>SNDK</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>profit</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="n">
+        <v>0.331205</v>
+      </c>
+      <c r="G3" s="13" t="n">
+        <v>903.13</v>
+      </c>
+      <c r="H3" s="13" t="n">
+        <v>1250.83</v>
+      </c>
+      <c r="I3" s="13" t="n"/>
+      <c r="J3" s="13">
+        <f>(H3-G3)*F3</f>
+        <v/>
+      </c>
+      <c r="K3" s="25">
+        <f>IF(G3&gt;0,(H3-G3)/G3,0)</f>
+        <v/>
+      </c>
+      <c r="L3" s="14">
+        <f>IF(AND(ISNUMBER(I3),G3-I3&lt;&gt;0),(H3-G3)/(G3-I3),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>BSE.NS</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>profit</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="G4" s="13" t="n">
+        <v>3415.5</v>
+      </c>
+      <c r="H4" s="13" t="n">
+        <v>3994.53</v>
+      </c>
+      <c r="I4" s="13" t="n"/>
+      <c r="J4" s="13">
+        <f>(H4-G4)*F4</f>
+        <v/>
+      </c>
+      <c r="K4" s="25">
+        <f>IF(G4&gt;0,(H4-G4)/G4,0)</f>
+        <v/>
+      </c>
+      <c r="L4" s="14">
+        <f>IF(AND(ISNUMBER(I4),G4-I4&lt;&gt;0),(H4-G4)/(G4-I4),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>KRN</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>loss</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>22</v>
+      </c>
+      <c r="G5" s="13" t="n">
+        <v>1310</v>
+      </c>
+      <c r="H5" s="13" t="n">
+        <v>1197.27</v>
+      </c>
+      <c r="I5" s="13" t="n"/>
+      <c r="J5" s="13">
+        <f>(H5-G5)*F5</f>
+        <v/>
+      </c>
+      <c r="K5" s="25">
+        <f>IF(G5&gt;0,(H5-G5)/G5,0)</f>
+        <v/>
+      </c>
+      <c r="L5" s="14">
+        <f>IF(AND(ISNUMBER(I5),G5-I5&lt;&gt;0),(H5-G5)/(G5-I5),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>CPRX</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>profit</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>7.178445</v>
+      </c>
+      <c r="G6" s="13" t="n">
+        <v>28.03</v>
+      </c>
+      <c r="H6" s="13" t="n">
+        <v>31.14</v>
+      </c>
+      <c r="I6" s="13" t="n"/>
+      <c r="J6" s="13">
+        <f>(H6-G6)*F6</f>
+        <v/>
+      </c>
+      <c r="K6" s="25">
+        <f>IF(G6&gt;0,(H6-G6)/G6,0)</f>
+        <v/>
+      </c>
+      <c r="L6" s="14">
+        <f>IF(AND(ISNUMBER(I6),G6-I6&lt;&gt;0),(H6-G6)/(G6-I6),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>ATHERENERG</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>profit</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="G7" s="13" t="n">
+        <v>960.4</v>
+      </c>
+      <c r="H7" s="13" t="n">
+        <v>979.5</v>
+      </c>
+      <c r="I7" s="13" t="n"/>
+      <c r="J7" s="13">
+        <f>(H7-G7)*F7</f>
+        <v/>
+      </c>
+      <c r="K7" s="25">
+        <f>IF(G7&gt;0,(H7-G7)/G7,0)</f>
+        <v/>
+      </c>
+      <c r="L7" s="14">
+        <f>IF(AND(ISNUMBER(I7),G7-I7&lt;&gt;0),(H7-G7)/(G7-I7),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>LRCX</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>scratch</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="G8" s="13" t="n">
+        <v>346.09</v>
+      </c>
+      <c r="H8" s="13" t="n">
+        <v>346</v>
+      </c>
+      <c r="I8" s="13" t="n"/>
+      <c r="J8" s="13">
+        <f>(H8-G8)*F8</f>
+        <v/>
+      </c>
+      <c r="K8" s="25">
+        <f>IF(G8&gt;0,(H8-G8)/G8,0)</f>
+        <v/>
+      </c>
+      <c r="L8" s="14">
+        <f>IF(AND(ISNUMBER(I8),G8-I8&lt;&gt;0),(H8-G8)/(G8-I8),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>DATAPATTNS</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>loss</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="G9" s="13" t="n">
+        <v>4805</v>
+      </c>
+      <c r="H9" s="13" t="n">
+        <v>4400</v>
+      </c>
+      <c r="I9" s="13" t="n"/>
+      <c r="J9" s="13">
+        <f>(H9-G9)*F9</f>
+        <v/>
+      </c>
+      <c r="K9" s="25">
+        <f>IF(G9&gt;0,(H9-G9)/G9,0)</f>
+        <v/>
+      </c>
+      <c r="L9" s="14">
+        <f>IF(AND(ISNUMBER(I9),G9-I9&lt;&gt;0),(H9-G9)/(G9-I9),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="n"/>
+      <c r="B10" s="5" t="n"/>
+      <c r="C10" s="5" t="n"/>
+      <c r="D10" s="5" t="n"/>
+      <c r="E10" s="5" t="n"/>
+      <c r="F10" s="5" t="n"/>
+      <c r="G10" s="5" t="n"/>
+      <c r="H10" s="5" t="n"/>
+      <c r="I10" s="5" t="n"/>
+      <c r="J10" s="5">
+        <f>IF(F10="","",(H10-G10)*F10)</f>
+        <v/>
+      </c>
+      <c r="K10" s="5">
+        <f>IF(G10="","",(H10-G10)/G10)</f>
+        <v/>
+      </c>
+      <c r="L10" s="5">
+        <f>IF(OR(I10="",G10-I10=0),"",(H10-G10)/(G10-I10))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="n"/>
+      <c r="B11" s="5" t="n"/>
+      <c r="C11" s="5" t="n"/>
+      <c r="D11" s="5" t="n"/>
+      <c r="E11" s="5" t="n"/>
+      <c r="F11" s="5" t="n"/>
+      <c r="G11" s="5" t="n"/>
+      <c r="H11" s="5" t="n"/>
+      <c r="I11" s="5" t="n"/>
+      <c r="J11" s="5">
+        <f>IF(F11="","",(H11-G11)*F11)</f>
+        <v/>
+      </c>
+      <c r="K11" s="5">
+        <f>IF(G11="","",(H11-G11)/G11)</f>
+        <v/>
+      </c>
+      <c r="L11" s="5">
+        <f>IF(OR(I11="",G11-I11=0),"",(H11-G11)/(G11-I11))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="n"/>
+      <c r="B12" s="5" t="n"/>
+      <c r="C12" s="5" t="n"/>
+      <c r="D12" s="5" t="n"/>
+      <c r="E12" s="5" t="n"/>
+      <c r="F12" s="5" t="n"/>
+      <c r="G12" s="5" t="n"/>
+      <c r="H12" s="5" t="n"/>
+      <c r="I12" s="5" t="n"/>
+      <c r="J12" s="5">
+        <f>IF(F12="","",(H12-G12)*F12)</f>
+        <v/>
+      </c>
+      <c r="K12" s="5">
+        <f>IF(G12="","",(H12-G12)/G12)</f>
+        <v/>
+      </c>
+      <c r="L12" s="5">
+        <f>IF(OR(I12="",G12-I12=0),"",(H12-G12)/(G12-I12))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="n"/>
+      <c r="B13" s="5" t="n"/>
+      <c r="C13" s="5" t="n"/>
+      <c r="D13" s="5" t="n"/>
+      <c r="E13" s="5" t="n"/>
+      <c r="F13" s="5" t="n"/>
+      <c r="G13" s="5" t="n"/>
+      <c r="H13" s="5" t="n"/>
+      <c r="I13" s="5" t="n"/>
+      <c r="J13" s="5">
+        <f>IF(F13="","",(H13-G13)*F13)</f>
+        <v/>
+      </c>
+      <c r="K13" s="5">
+        <f>IF(G13="","",(H13-G13)/G13)</f>
+        <v/>
+      </c>
+      <c r="L13" s="5">
+        <f>IF(OR(I13="",G13-I13=0),"",(H13-G13)/(G13-I13))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="n"/>
+      <c r="B14" s="5" t="n"/>
+      <c r="C14" s="5" t="n"/>
+      <c r="D14" s="5" t="n"/>
+      <c r="E14" s="5" t="n"/>
+      <c r="F14" s="5" t="n"/>
+      <c r="G14" s="5" t="n"/>
+      <c r="H14" s="5" t="n"/>
+      <c r="I14" s="5" t="n"/>
+      <c r="J14" s="5">
+        <f>IF(F14="","",(H14-G14)*F14)</f>
+        <v/>
+      </c>
+      <c r="K14" s="5">
+        <f>IF(G14="","",(H14-G14)/G14)</f>
+        <v/>
+      </c>
+      <c r="L14" s="5">
+        <f>IF(OR(I14="",G14-I14=0),"",(H14-G14)/(G14-I14))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="n"/>
+      <c r="B15" s="5" t="n"/>
+      <c r="C15" s="5" t="n"/>
+      <c r="D15" s="5" t="n"/>
+      <c r="E15" s="5" t="n"/>
+      <c r="F15" s="5" t="n"/>
+      <c r="G15" s="5" t="n"/>
+      <c r="H15" s="5" t="n"/>
+      <c r="I15" s="5" t="n"/>
+      <c r="J15" s="5">
+        <f>IF(F15="","",(H15-G15)*F15)</f>
+        <v/>
+      </c>
+      <c r="K15" s="5">
+        <f>IF(G15="","",(H15-G15)/G15)</f>
+        <v/>
+      </c>
+      <c r="L15" s="5">
+        <f>IF(OR(I15="",G15-I15=0),"",(H15-G15)/(G15-I15))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="n"/>
+      <c r="B16" s="5" t="n"/>
+      <c r="C16" s="5" t="n"/>
+      <c r="D16" s="5" t="n"/>
+      <c r="E16" s="5" t="n"/>
+      <c r="F16" s="5" t="n"/>
+      <c r="G16" s="5" t="n"/>
+      <c r="H16" s="5" t="n"/>
+      <c r="I16" s="5" t="n"/>
+      <c r="J16" s="5">
+        <f>IF(F16="","",(H16-G16)*F16)</f>
+        <v/>
+      </c>
+      <c r="K16" s="5">
+        <f>IF(G16="","",(H16-G16)/G16)</f>
+        <v/>
+      </c>
+      <c r="L16" s="5">
+        <f>IF(OR(I16="",G16-I16=0),"",(H16-G16)/(G16-I16))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="n"/>
+      <c r="B17" s="5" t="n"/>
+      <c r="C17" s="5" t="n"/>
+      <c r="D17" s="5" t="n"/>
+      <c r="E17" s="5" t="n"/>
+      <c r="F17" s="5" t="n"/>
+      <c r="G17" s="5" t="n"/>
+      <c r="H17" s="5" t="n"/>
+      <c r="I17" s="5" t="n"/>
+      <c r="J17" s="5">
+        <f>IF(F17="","",(H17-G17)*F17)</f>
+        <v/>
+      </c>
+      <c r="K17" s="5">
+        <f>IF(G17="","",(H17-G17)/G17)</f>
+        <v/>
+      </c>
+      <c r="L17" s="5">
+        <f>IF(OR(I17="",G17-I17=0),"",(H17-G17)/(G17-I17))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="n"/>
+      <c r="B18" s="5" t="n"/>
+      <c r="C18" s="5" t="n"/>
+      <c r="D18" s="5" t="n"/>
+      <c r="E18" s="5" t="n"/>
+      <c r="F18" s="5" t="n"/>
+      <c r="G18" s="5" t="n"/>
+      <c r="H18" s="5" t="n"/>
+      <c r="I18" s="5" t="n"/>
+      <c r="J18" s="5">
+        <f>IF(F18="","",(H18-G18)*F18)</f>
+        <v/>
+      </c>
+      <c r="K18" s="5">
+        <f>IF(G18="","",(H18-G18)/G18)</f>
+        <v/>
+      </c>
+      <c r="L18" s="5">
+        <f>IF(OR(I18="",G18-I18=0),"",(H18-G18)/(G18-I18))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="n"/>
+      <c r="B19" s="5" t="n"/>
+      <c r="C19" s="5" t="n"/>
+      <c r="D19" s="5" t="n"/>
+      <c r="E19" s="5" t="n"/>
+      <c r="F19" s="5" t="n"/>
+      <c r="G19" s="5" t="n"/>
+      <c r="H19" s="5" t="n"/>
+      <c r="I19" s="5" t="n"/>
+      <c r="J19" s="5">
+        <f>IF(F19="","",(H19-G19)*F19)</f>
+        <v/>
+      </c>
+      <c r="K19" s="5">
+        <f>IF(G19="","",(H19-G19)/G19)</f>
+        <v/>
+      </c>
+      <c r="L19" s="5">
+        <f>IF(OR(I19="",G19-I19=0),"",(H19-G19)/(G19-I19))</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:L1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F32"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="26" t="inlineStr">
+        <is>
+          <t>POSITION SIZING &amp; R:R CALCULATOR</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Yellow = type your numbers. Blue = auto-computed. Mirrors rr_calc.py.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Trade Inputs</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="27" t="inlineStr">
+        <is>
+          <t>Entry price</t>
+        </is>
+      </c>
+      <c r="B5" s="28" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="27" t="inlineStr">
+        <is>
+          <t>Stop loss</t>
+        </is>
+      </c>
+      <c r="B6" s="28" t="n">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="27" t="inlineStr">
+        <is>
+          <t>Account / sleeve ₹</t>
+        </is>
+      </c>
+      <c r="B7" s="29" t="n">
+        <v>263453</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="27" t="inlineStr">
+        <is>
+          <t>Risk budget %</t>
+        </is>
+      </c>
+      <c r="B8" s="30" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Position Sizing (from risk budget)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="27" t="inlineStr">
+        <is>
+          <t>Risk per share</t>
+        </is>
+      </c>
+      <c r="B11" s="31">
+        <f>B5-B6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="27" t="inlineStr">
+        <is>
+          <t>Risk % of entry</t>
+        </is>
+      </c>
+      <c r="B12" s="32">
+        <f>(B5-B6)/B5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="27" t="inlineStr">
+        <is>
+          <t>Max ₹ at risk</t>
+        </is>
+      </c>
+      <c r="B13" s="33">
+        <f>B7*B8/100</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="27" t="inlineStr">
+        <is>
+          <t>Max shares</t>
+        </is>
+      </c>
+      <c r="B14" s="33">
+        <f>IF(B11&gt;0,FLOOR(B13/B11,1),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="27" t="inlineStr">
+        <is>
+          <t>Capital required</t>
+        </is>
+      </c>
+      <c r="B15" s="33">
+        <f>B14*B5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="27" t="inlineStr">
+        <is>
+          <t>% of sleeve deployed</t>
+        </is>
+      </c>
+      <c r="B16" s="34">
+        <f>IF(B7&gt;0,B15/B7,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>25-50-25 Pyramid Split (of max shares)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="27" t="inlineStr">
+        <is>
+          <t>T1 pilot (25%)</t>
+        </is>
+      </c>
+      <c r="B19" s="33">
+        <f>FLOOR(B14*0.25,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="27" t="inlineStr">
+        <is>
+          <t>T2 core (50%)</t>
+        </is>
+      </c>
+      <c r="B20" s="33">
+        <f>FLOOR(B14*0.5,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="27" t="inlineStr">
+        <is>
+          <t>T3 final (25%)</t>
+        </is>
+      </c>
+      <c r="B21" s="33">
+        <f>B14-B19-B20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Targets &amp; Weighted R:R (edit prices + % to sell)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="35" t="inlineStr">
+        <is>
+          <t>Target</t>
+        </is>
+      </c>
+      <c r="B24" s="35" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+      <c r="C24" s="35" t="inlineStr">
+        <is>
+          <t>% of position</t>
+        </is>
+      </c>
+      <c r="D24" s="35" t="inlineStr">
+        <is>
+          <t>R:R</t>
+        </is>
+      </c>
+      <c r="E24" s="35" t="inlineStr">
+        <is>
+          <t>Reward %</t>
+        </is>
+      </c>
+      <c r="F24" s="35" t="inlineStr">
+        <is>
+          <t>P&amp;L ₹ (at max shares)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="27" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="B25" s="28" t="n">
+        <v>110</v>
+      </c>
+      <c r="C25" s="36" t="n">
+        <v>33</v>
+      </c>
+      <c r="D25" s="37">
+        <f>IF($B$5-$B$6&gt;0,(B25-$B$5)/($B$5-$B$6),0)</f>
+        <v/>
+      </c>
+      <c r="E25" s="34">
+        <f>(B25-$B$5)/$B$5</f>
+        <v/>
+      </c>
+      <c r="F25" s="33">
+        <f>(B25-$B$5)*FLOOR($B$14*C25/100,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="27" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="B26" s="28" t="n">
+        <v>120</v>
+      </c>
+      <c r="C26" s="36" t="n">
+        <v>33</v>
+      </c>
+      <c r="D26" s="37">
+        <f>IF($B$5-$B$6&gt;0,(B26-$B$5)/($B$5-$B$6),0)</f>
+        <v/>
+      </c>
+      <c r="E26" s="34">
+        <f>(B26-$B$5)/$B$5</f>
+        <v/>
+      </c>
+      <c r="F26" s="33">
+        <f>(B26-$B$5)*FLOOR($B$14*C26/100,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="27" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="B27" s="28" t="n">
+        <v>135</v>
+      </c>
+      <c r="C27" s="36" t="n">
+        <v>34</v>
+      </c>
+      <c r="D27" s="37">
+        <f>IF($B$5-$B$6&gt;0,(B27-$B$5)/($B$5-$B$6),0)</f>
+        <v/>
+      </c>
+      <c r="E27" s="34">
+        <f>(B27-$B$5)/$B$5</f>
+        <v/>
+      </c>
+      <c r="F27" s="33">
+        <f>(B27-$B$5)*FLOOR($B$14*C27/100,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="38" t="inlineStr">
+        <is>
+          <t>Weighted avg R:R</t>
+        </is>
+      </c>
+      <c r="D28" s="37">
+        <f>IF(SUM(C25:C27)&gt;0,SUMPRODUCT(D25:D27,C25:C27)/SUM(C25:C27),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="38" t="inlineStr">
+        <is>
+          <t>Avg exit price</t>
+        </is>
+      </c>
+      <c r="B29" s="31">
+        <f>IF(SUM(C25:C27)&gt;0,SUMPRODUCT(B25:B27,C25:C27)/SUM(C25:C27),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="38" t="inlineStr">
+        <is>
+          <t>Full-run P&amp;L ₹</t>
+        </is>
+      </c>
+      <c r="B30" s="33">
+        <f>SUM(F25:F27)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="38" t="inlineStr">
+        <is>
+          <t>Payoff ratio (win/loss)</t>
+        </is>
+      </c>
+      <c r="B31" s="37">
+        <f>IF(B13&gt;0,B30/B13,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="38" t="inlineStr">
+        <is>
+          <t>Break-even win rate</t>
+        </is>
+      </c>
+      <c r="B32" s="34">
+        <f>IF(B31&gt;0,1/(1+B31),0)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A23:F23"/>
+    <mergeCell ref="A18:D18"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:J12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -3890,7 +4974,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Father's Portfolio — as of 2026-08-11 (LTP refreshed on generation)</t>
+          <t>Father's Portfolio — as of 2026-08-12 (LTP refreshed on generation)</t>
         </is>
       </c>
     </row>
@@ -3978,7 +5062,7 @@
       <c r="I3" s="21" t="n">
         <v>30.59031517163864</v>
       </c>
-      <c r="J3" s="25" t="inlineStr">
+      <c r="J3" s="39" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -4023,16 +5107,16 @@
       <c r="I5" s="23" t="n">
         <v>-23.05421294278932</v>
       </c>
-      <c r="J5" s="26" t="inlineStr">
-        <is>
-          <t>SELL_PLANNED</t>
+      <c r="J5" s="40" t="inlineStr">
+        <is>
+          <t>HOLD_FOR_TLH</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>↳ Exit planned at ~-23% loss. Est. proceeds ~38L at current prices</t>
+          <t>↳ Deliberate hold: exit to be timed against realized GAINS elsewhere for tax-loss harvesting (~11L loss available to offset). Not a conviction hold.</t>
         </is>
       </c>
     </row>
@@ -4048,7 +5132,7 @@
         </is>
       </c>
       <c r="C7" s="5" t="n">
-        <v>600</v>
+        <v>0</v>
       </c>
       <c r="D7" s="13" t="n">
         <v>2428.21</v>
@@ -4056,28 +5140,20 @@
       <c r="E7" s="13" t="n">
         <v>2005</v>
       </c>
-      <c r="F7" s="6" t="n">
-        <v>1203000</v>
-      </c>
-      <c r="G7" s="6" t="n">
-        <v>1456928.3</v>
-      </c>
-      <c r="H7" s="22" t="n">
-        <v>-253928.3</v>
-      </c>
-      <c r="I7" s="23" t="n">
-        <v>-17.42901829829238</v>
-      </c>
-      <c r="J7" s="27" t="inlineStr">
-        <is>
-          <t>MOSTLY_SOLD</t>
+      <c r="F7" s="6" t="n"/>
+      <c r="G7" s="6" t="n"/>
+      <c r="H7" s="6" t="n"/>
+      <c r="I7" s="5" t="n"/>
+      <c r="J7" s="41" t="inlineStr">
+        <is>
+          <t>SOLD</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>↳ Sold almost entirely per Vishesh. Snapshot qty 600 predates sale — update residual</t>
+          <t>↳ Fully exited — all 600 units sold Aug 2026. Realized loss ~₹2.5L (confirm exact from contract note)</t>
         </is>
       </c>
     </row>
@@ -4088,13 +5164,13 @@
         </is>
       </c>
       <c r="F9" s="9" t="n">
-        <v>7559650</v>
+        <v>6356650</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>8350431.37</v>
+        <v>6893503.07</v>
       </c>
       <c r="H9" s="12" t="n">
-        <v>-790781.3700000001</v>
+        <v>-536853.0700000003</v>
       </c>
     </row>
     <row r="11">

</xml_diff>

<commit_message>
Add dormant/set-and-forget US account; fix cross-account price cache leak
- New us_holdings_dormant bucket: 7 ETFs (QQQM, SMH, VDE, VEU, VFH, VOO,
  VTI), separate account not actively traded — overlaps in ticker with
  the active Alpaca account but kept additive, not merged.
- build_us_sheet refactored to accept multiple (account_label, holdings)
  pairs on one tab, each with its own subtotal, rolling into one grand
  total for the Dashboard.
- Bug fix: Prices.get() was caching "cached" (cost-basis fallback) results
  by symbol alone, so the same ticker held in two accounts at different
  avg prices leaked one account's cost basis into the other's row. Only
  "live"/"override" results (genuinely universal per symbol) are now
  cached; "cached" fallback is always recomputed from the caller's own
  cached_ltp.

https://claude.ai/code/session_01HhF36NsLiVFyxhhXe4S24m
</commit_message>
<xml_diff>
--- a/examples/swing_monitor/Portfolio_Tracker.xlsx
+++ b/examples/swing_monitor/Portfolio_Tracker.xlsx
@@ -575,7 +575,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-12 12:34  |  USD/INR 95.0  |  prices: override file (2026-08-12T10:29:00+00:00), yfinance off</t>
+          <t>Generated 2026-08-12 12:42  |  USD/INR 95.0  |  prices: override file (2026-08-12T10:29:00+00:00), yfinance off</t>
         </is>
       </c>
     </row>
@@ -663,10 +663,10 @@
         </is>
       </c>
       <c r="B9" s="6" t="n">
-        <v>896077.1993590571</v>
+        <v>1153488.284461557</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>896077.1993590571</v>
+        <v>1153488.284461557</v>
       </c>
       <c r="D9" s="7" t="n">
         <v>0</v>
@@ -695,13 +695,13 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>3046000.389359057</v>
+        <v>3303411.474461557</v>
       </c>
       <c r="C11" s="9" t="n">
-        <v>3236389.879359057</v>
+        <v>3493800.964461558</v>
       </c>
       <c r="D11" s="10" t="n">
-        <v>190389.4899999998</v>
+        <v>190389.4900000002</v>
       </c>
     </row>
     <row r="13">
@@ -2419,7 +2419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I32"/>
+  <dimension ref="A1:I46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2436,7 +2436,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>US ETFs</t>
+          <t>Alpaca (active) — ETFs</t>
         </is>
       </c>
     </row>
@@ -2945,7 +2945,7 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>US Stocks</t>
+          <t>Alpaca (active) — Stocks</t>
         </is>
       </c>
     </row>
@@ -3486,10 +3486,342 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="B34" s="8" t="inlineStr">
+        <is>
+          <t>Alpaca (active) subtotal</t>
+        </is>
+      </c>
+      <c r="E34" s="9" t="n">
+        <v>896077.1993590571</v>
+      </c>
+      <c r="F34" s="9" t="n">
+        <v>896077.1993590571</v>
+      </c>
+      <c r="G34" s="20" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>TBD — confirm account/broker name (set-and-forget) — ETFs</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Symbol</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>Price $</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>Value ₹</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>Invested ₹</t>
+        </is>
+      </c>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>P&amp;L ₹</t>
+        </is>
+      </c>
+      <c r="H37" s="4" t="inlineStr">
+        <is>
+          <t>P&amp;L %</t>
+        </is>
+      </c>
+      <c r="I37" s="4" t="inlineStr">
+        <is>
+          <t>Price Src</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>QQQM</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>Invesco NASDAQ 100 ETF</t>
+        </is>
+      </c>
+      <c r="C38" s="24" t="n">
+        <v>2.02555</v>
+      </c>
+      <c r="D38" s="13" t="n">
+        <v>297.65</v>
+      </c>
+      <c r="E38" s="6" t="n">
+        <v>57275.97096249999</v>
+      </c>
+      <c r="F38" s="6" t="n">
+        <v>57275.97096249999</v>
+      </c>
+      <c r="G38" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H38" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I38" s="17" t="inlineStr">
+        <is>
+          <t>cached</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>SMH</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>VanEck Semiconductor ETF</t>
+        </is>
+      </c>
+      <c r="C39" s="24" t="n">
+        <v>0.44718</v>
+      </c>
+      <c r="D39" s="13" t="n">
+        <v>585.98</v>
+      </c>
+      <c r="E39" s="6" t="n">
+        <v>24893.660958</v>
+      </c>
+      <c r="F39" s="6" t="n">
+        <v>24893.660958</v>
+      </c>
+      <c r="G39" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H39" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I39" s="17" t="inlineStr">
+        <is>
+          <t>cached</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>VDE</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>Vanguard Energy ETF</t>
+        </is>
+      </c>
+      <c r="C40" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="D40" s="13" t="n">
+        <v>167.88</v>
+      </c>
+      <c r="E40" s="6" t="n">
+        <v>15948.6</v>
+      </c>
+      <c r="F40" s="6" t="n">
+        <v>15948.6</v>
+      </c>
+      <c r="G40" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H40" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I40" s="17" t="inlineStr">
+        <is>
+          <t>cached</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>VEU</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>Vanguard FTSE All-World ex-US ETF</t>
+        </is>
+      </c>
+      <c r="C41" s="24" t="n">
+        <v>3.7037</v>
+      </c>
+      <c r="D41" s="13" t="n">
+        <v>82.44</v>
+      </c>
+      <c r="E41" s="6" t="n">
+        <v>29006.63766</v>
+      </c>
+      <c r="F41" s="6" t="n">
+        <v>29006.63766</v>
+      </c>
+      <c r="G41" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H41" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I41" s="17" t="inlineStr">
+        <is>
+          <t>cached</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>VFH</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>Vanguard Financials ETF</t>
+        </is>
+      </c>
+      <c r="C42" s="24" t="n">
+        <v>2.10229</v>
+      </c>
+      <c r="D42" s="13" t="n">
+        <v>127.8</v>
+      </c>
+      <c r="E42" s="6" t="n">
+        <v>25523.90289</v>
+      </c>
+      <c r="F42" s="6" t="n">
+        <v>25523.90289</v>
+      </c>
+      <c r="G42" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H42" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I42" s="17" t="inlineStr">
+        <is>
+          <t>cached</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>VOO</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>Vanguard S&amp;P 500 ETF</t>
+        </is>
+      </c>
+      <c r="C43" s="24" t="n">
+        <v>1.17292</v>
+      </c>
+      <c r="D43" s="13" t="n">
+        <v>684.38</v>
+      </c>
+      <c r="E43" s="6" t="n">
+        <v>76258.684012</v>
+      </c>
+      <c r="F43" s="6" t="n">
+        <v>76258.684012</v>
+      </c>
+      <c r="G43" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H43" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I43" s="17" t="inlineStr">
+        <is>
+          <t>cached</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>VTI</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>Vanguard Total Stock Market ETF</t>
+        </is>
+      </c>
+      <c r="C44" s="24" t="n">
+        <v>0.8284</v>
+      </c>
+      <c r="D44" s="13" t="n">
+        <v>362.19</v>
+      </c>
+      <c r="E44" s="6" t="n">
+        <v>28503.62862</v>
+      </c>
+      <c r="F44" s="6" t="n">
+        <v>28503.62862</v>
+      </c>
+      <c r="G44" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H44" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I44" s="17" t="inlineStr">
+        <is>
+          <t>cached</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" s="8" t="inlineStr">
+        <is>
+          <t>TBD — confirm account/broker name (set-and-forget) subtotal</t>
+        </is>
+      </c>
+      <c r="E46" s="9" t="n">
+        <v>257411.0851025</v>
+      </c>
+      <c r="F46" s="9" t="n">
+        <v>257411.0851025</v>
+      </c>
+      <c r="G46" s="20" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A17:I17"/>
+    <mergeCell ref="A36:I36"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Gate NETWEB Core/Final tranches on market regime — Nifty 50 lost 21D EMA
Regime check (M in CANSLIM) using user-supplied Nifty 50/500 MA charts:
Nifty 50 price 24,202 is below 10D, 21D, 150D, AND 200D — only above the
50D. The codified watchlist rule "exit longs if loses 21D EMA" has fired.
Nifty 500 is weaker but not broken (only below its 10D EMA). RS vs Nasdaq
at 11 (bottom decile), falling.

NETWEB qty pulled back from 24 (full plan) to 6 (pilot only). Core (12sh)
and Final (6sh) tranches now explicitly gated on Nifty 50 reclaiming its
21D EMA, or a recognized follow-through day — not on the stock's own
strength alone. Added NIFTY500 (^CRSLDX) as a second regime gauge, more
relevant to mid/small-cap names than the large-cap-heavy Nifty 50.

https://claude.ai/code/session_01HhF36NsLiVFyxhhXe4S24m
</commit_message>
<xml_diff>
--- a/examples/swing_monitor/Portfolio_Tracker.xlsx
+++ b/examples/swing_monitor/Portfolio_Tracker.xlsx
@@ -576,7 +576,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-18 06:35  |  USD/INR 95.0  |  prices: override file (2026-08-12T10:29:00+00:00), yfinance off</t>
+          <t>Generated 2026-08-18 08:53  |  USD/INR 95.0  |  prices: override file (2026-08-12T10:29:00+00:00), yfinance off</t>
         </is>
       </c>
     </row>
@@ -3834,7 +3834,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I28"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3923,7 +3923,7 @@
         </is>
       </c>
       <c r="B6" s="25" t="n">
-        <v>24</v>
+        <v>6</v>
       </c>
       <c r="C6" s="25" t="n">
         <v>5314.05</v>
@@ -3943,7 +3943,7 @@
         </is>
       </c>
       <c r="H6" s="25" t="n">
-        <v>11737.2</v>
+        <v>2934.300000000001</v>
       </c>
       <c r="I6" s="25" t="inlineStr">
         <is>
@@ -3954,7 +3954,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>↳ NETWEB: Pilot 6sh now (within 5240-5500 buy range). Core 12sh add on decisive breakout &gt;5500 on above-avg volume, OR 3-5 days holding &gt;5244. Final 6sh at/after T1 (5800), pullback to 10D EMA holds. Stop to breakeven after Core fills; trail 10D/21D EMA after Final.</t>
+          <t>↳ NETWEB: PILOT 6sh now (within 5240-5500 buy range) — stock-specific strength justifies a toe in despite regime caution. CORE 12sh GATED: only after Nifty 50 reclaims 21D EMA (24,326) and ideally 150D SMA (24,294), OR a recognized O'Neil follow-through day. Do not add Core on the stock's own strength alone while the index rule is active. FINAL 6sh at/after T1 (5800), pullback to 10D EMA holds, market regime still confirming. Stop to breakeven after Core fills; trail 10D/21D EMA after Final. If Nifty 50 closes below 50D SMA (24,124), tighten pilot stop rather than average in.</t>
         </is>
       </c>
     </row>
@@ -4134,103 +4134,88 @@
       <c r="C17" s="5" t="inlineStr"/>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Regime gauge — exit longs if loses 21D EMA</t>
+          <t>RULE FIRED 2026-08-14: price 24,202 lost 21D EMA (24,326) AND 10D EMA (24,374) AND 150D SMA (24,294) AND 200D SMA (24,714) — only above 50D (24,124). Do not deploy new swing longs beyond pilot size until 21D EMA reclaimed.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>NIFTY500</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr"/>
       <c r="C18" s="5" t="inlineStr"/>
       <c r="D18" s="2" t="inlineStr">
         <is>
+          <t>Weaker but not broken: price 23,508 below 10D EMA (23,591) only, still above 21D/50D/150D/200D. Broader-market gauge for mid/small-cap names (more relevant than Nifty50 for names like NETWEB). RS vs Nasdaq at 11 (bottom decile), falling.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr"/>
+      <c r="C19" s="5" t="inlineStr"/>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
           <t>US regime gauge — chip selloff in progress, watch for follow-through distribution</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>Closed Trade Journal</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B21" s="4" t="inlineStr">
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>Result</t>
         </is>
       </c>
-      <c r="C21" s="4" t="inlineStr">
+      <c r="C22" s="4" t="inlineStr">
         <is>
           <t>Avg Entry</t>
         </is>
       </c>
-      <c r="D21" s="4" t="inlineStr">
+      <c r="D22" s="4" t="inlineStr">
         <is>
           <t>Avg Exit</t>
         </is>
       </c>
-      <c r="E21" s="4" t="inlineStr">
+      <c r="E22" s="4" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
       </c>
-      <c r="F21" s="4" t="inlineStr">
+      <c r="F22" s="4" t="inlineStr">
         <is>
           <t>P&amp;L %</t>
         </is>
       </c>
-      <c r="G21" s="4" t="inlineStr">
+      <c r="G22" s="4" t="inlineStr">
         <is>
           <t>Hold Days</t>
         </is>
       </c>
-      <c r="H21" s="4" t="inlineStr"/>
-      <c r="I21" s="4" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="5" t="inlineStr">
-        <is>
-          <t>SNDK</t>
-        </is>
-      </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>profit</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="n">
-        <v>903.13</v>
-      </c>
-      <c r="D22" s="5" t="n">
-        <v>1250.83</v>
-      </c>
-      <c r="E22" s="5" t="inlineStr">
-        <is>
-          <t>$113</t>
-        </is>
-      </c>
-      <c r="F22" s="21" t="n">
-        <v>37.7</v>
-      </c>
-      <c r="G22" s="5" t="n">
-        <v>35</v>
-      </c>
+      <c r="H22" s="4" t="inlineStr"/>
+      <c r="I22" s="4" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>BSE.NS</t>
+          <t>SNDK</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
@@ -4239,85 +4224,85 @@
         </is>
       </c>
       <c r="C23" s="5" t="n">
-        <v>3415.5</v>
+        <v>903.13</v>
       </c>
       <c r="D23" s="5" t="n">
-        <v>3994.53</v>
+        <v>1250.83</v>
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>₹4,632</t>
+          <t>$113</t>
         </is>
       </c>
       <c r="F23" s="21" t="n">
-        <v>17</v>
+        <v>37.7</v>
       </c>
       <c r="G23" s="5" t="n">
-        <v>48</v>
+        <v>35</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>KRN</t>
+          <t>BSE.NS</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>loss</t>
+          <t>profit</t>
         </is>
       </c>
       <c r="C24" s="5" t="n">
-        <v>1310</v>
+        <v>3415.5</v>
       </c>
       <c r="D24" s="5" t="n">
-        <v>1197.27</v>
+        <v>3994.53</v>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>₹-2,480</t>
-        </is>
-      </c>
-      <c r="F24" s="23" t="n">
-        <v>-8.6</v>
+          <t>₹4,632</t>
+        </is>
+      </c>
+      <c r="F24" s="21" t="n">
+        <v>17</v>
       </c>
       <c r="G24" s="5" t="n">
-        <v>9</v>
+        <v>48</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>CPRX</t>
+          <t>KRN</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>profit</t>
+          <t>loss</t>
         </is>
       </c>
       <c r="C25" s="5" t="n">
-        <v>28.03</v>
+        <v>1310</v>
       </c>
       <c r="D25" s="5" t="n">
-        <v>31.14</v>
+        <v>1197.27</v>
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>$21</t>
-        </is>
-      </c>
-      <c r="F25" s="21" t="n">
-        <v>10.4</v>
+          <t>₹-2,480</t>
+        </is>
+      </c>
+      <c r="F25" s="23" t="n">
+        <v>-8.6</v>
       </c>
       <c r="G25" s="5" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>ATHERENERG</t>
+          <t>CPRX</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
@@ -4326,81 +4311,111 @@
         </is>
       </c>
       <c r="C26" s="5" t="n">
-        <v>960.4</v>
+        <v>28.03</v>
       </c>
       <c r="D26" s="5" t="n">
-        <v>979.5</v>
+        <v>31.14</v>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>₹134</t>
+          <t>$21</t>
         </is>
       </c>
       <c r="F26" s="21" t="n">
-        <v>2</v>
+        <v>10.4</v>
       </c>
       <c r="G26" s="5" t="n">
-        <v>37</v>
+        <v>14</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>LRCX</t>
+          <t>ATHERENERG</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>scratch</t>
+          <t>profit</t>
         </is>
       </c>
       <c r="C27" s="5" t="n">
-        <v>346.09</v>
+        <v>960.4</v>
       </c>
       <c r="D27" s="5" t="n">
-        <v>346</v>
+        <v>979.5</v>
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>$-0</t>
-        </is>
-      </c>
-      <c r="F27" s="23" t="n">
-        <v>-0.03</v>
+          <t>₹134</t>
+        </is>
+      </c>
+      <c r="F27" s="21" t="n">
+        <v>2</v>
       </c>
       <c r="G27" s="5" t="n">
-        <v>27</v>
+        <v>37</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
+          <t>LRCX</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>scratch</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="n">
+        <v>346.09</v>
+      </c>
+      <c r="D28" s="5" t="n">
+        <v>346</v>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>$-0</t>
+        </is>
+      </c>
+      <c r="F28" s="23" t="n">
+        <v>-0.03</v>
+      </c>
+      <c r="G28" s="5" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
           <t>DATAPATTNS</t>
         </is>
       </c>
-      <c r="B28" s="5" t="inlineStr">
+      <c r="B29" s="5" t="inlineStr">
         <is>
           <t>loss</t>
         </is>
       </c>
-      <c r="C28" s="5" t="n">
+      <c r="C29" s="5" t="n">
         <v>4805</v>
       </c>
-      <c r="D28" s="5" t="n">
+      <c r="D29" s="5" t="n">
         <v>4400</v>
       </c>
-      <c r="E28" s="5" t="inlineStr">
+      <c r="E29" s="5" t="inlineStr">
         <is>
           <t>₹-4,050</t>
         </is>
       </c>
-      <c r="F28" s="23" t="n">
+      <c r="F29" s="23" t="n">
         <v>-8.4</v>
       </c>
-      <c r="G28" s="5" t="n"/>
+      <c r="G29" s="5" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="14">
+    <mergeCell ref="D19:I19"/>
     <mergeCell ref="A7:I7"/>
     <mergeCell ref="D11:I11"/>
     <mergeCell ref="D13:I13"/>
@@ -4412,7 +4427,7 @@
     <mergeCell ref="D12:I12"/>
     <mergeCell ref="D16:I16"/>
     <mergeCell ref="A4:I4"/>
-    <mergeCell ref="A20:I20"/>
+    <mergeCell ref="A21:I21"/>
     <mergeCell ref="D15:I15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Log NETWEB fill: 6sh @ 5,348, tactical stop 5,085
Entered pilot tranche at ₹5,348. Working stop set to 5,085 (SL-M trigger,
~7pt buffer below entry-day low 5,092) — a tighter, tactical day-1-low
stop rather than the original 8%-below-pivot structural stop (4,825,
kept as stop_structural for reference). Risk ₹1,578 (0.13% of growth
sleeve). Core/Final tranches remain regime-gated on Nifty 50 reclaiming
its 21D EMA.

https://claude.ai/code/session_01HhF36NsLiVFyxhhXe4S24m
</commit_message>
<xml_diff>
--- a/examples/swing_monitor/Portfolio_Tracker.xlsx
+++ b/examples/swing_monitor/Portfolio_Tracker.xlsx
@@ -105,11 +105,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FEF3C7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00FEF9C3"/>
       </patternFill>
     </fill>
@@ -121,6 +116,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00DCFCE7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF3C7"/>
       </patternFill>
     </fill>
     <fill>
@@ -146,7 +146,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -174,23 +174,22 @@
     <xf numFmtId="3" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="169" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -576,7 +575,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-18 08:53  |  USD/INR 95.0  |  prices: override file (2026-08-12T10:29:00+00:00), yfinance off</t>
+          <t>Generated 2026-08-18 09:06  |  USD/INR 95.0  |  prices: override file (2026-08-12T10:29:00+00:00), yfinance off</t>
         </is>
       </c>
     </row>
@@ -3834,7 +3833,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:I28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3856,366 +3855,386 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>No open positions — flat.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>Entry</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>LTP</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>Next Target</t>
+        </is>
+      </c>
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>P&amp;L %</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>Risk ₹</t>
+        </is>
+      </c>
+      <c r="I2" s="4" t="inlineStr">
+        <is>
+          <t>Src</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>NETWEB</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="C3" s="5" t="n">
+        <v>5348</v>
+      </c>
+      <c r="D3" s="5" t="n">
+        <v>5314.05</v>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>5085</v>
+      </c>
+      <c r="F3" s="5" t="n">
+        <v>5800</v>
+      </c>
+      <c r="G3" s="23" t="n">
+        <v>-0.6348167539267036</v>
+      </c>
+      <c r="H3" s="5" t="n">
+        <v>1578</v>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>override</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Planned Positions (staged, not filled)</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>No planned positions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Watchlist / Planned Entries</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>Plan Qty</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>Pilot Entry</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>LTP</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Trigger</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>Stop</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>Pivot</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>Dist to Buy Zone</t>
-        </is>
-      </c>
-      <c r="H5" s="4" t="inlineStr">
-        <is>
-          <t>Risk ₹ (full)</t>
-        </is>
-      </c>
-      <c r="I5" s="4" t="inlineStr">
-        <is>
-          <t>Src</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="25" t="inlineStr">
-        <is>
-          <t>NETWEB</t>
-        </is>
-      </c>
-      <c r="B6" s="25" t="n">
-        <v>6</v>
-      </c>
-      <c r="C6" s="25" t="n">
-        <v>5314.05</v>
-      </c>
-      <c r="D6" s="25" t="n">
-        <v>5314.05</v>
-      </c>
-      <c r="E6" s="25" t="n">
-        <v>4825</v>
-      </c>
-      <c r="F6" s="25" t="n">
-        <v>5244</v>
-      </c>
-      <c r="G6" s="25" t="inlineStr">
-        <is>
-          <t>IN ZONE</t>
-        </is>
-      </c>
-      <c r="H6" s="25" t="n">
-        <v>2934.300000000001</v>
-      </c>
-      <c r="I6" s="25" t="inlineStr">
-        <is>
-          <t>override</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>↳ NETWEB: PILOT 6sh now (within 5240-5500 buy range) — stock-specific strength justifies a toe in despite regime caution. CORE 12sh GATED: only after Nifty 50 reclaims 21D EMA (24,326) and ideally 150D SMA (24,294), OR a recognized O'Neil follow-through day. Do not add Core on the stock's own strength alone while the index rule is active. FINAL 6sh at/after T1 (5800), pullback to 10D EMA holds, market regime still confirming. Stop to breakeven after Core fills; trail 10D/21D EMA after Final. If Nifty 50 closes below 50D SMA (24,124), tighten pilot stop rather than average in.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>Watchlist / Planned Entries</t>
-        </is>
-      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr"/>
+      <c r="F9" s="4" t="inlineStr"/>
+      <c r="G9" s="4" t="inlineStr"/>
+      <c r="H9" s="4" t="inlineStr"/>
+      <c r="I9" s="4" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Ticker</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>Trigger</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>Stop</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="inlineStr"/>
-      <c r="F10" s="4" t="inlineStr"/>
-      <c r="G10" s="4" t="inlineStr"/>
-      <c r="H10" s="4" t="inlineStr"/>
-      <c r="I10" s="4" t="inlineStr"/>
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>POLYCAB</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>₹9690 reclaim</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>₹9265</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>A- setup. Fresh box breakout to ATH 10,126, now pulling back. Enter 25% pilot on reclaim of 10D EMA 9,690. Add 50% above 10,126. Invalidate below 50D 9,265.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>POLYCAB</t>
+          <t>ACUTAAS</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>₹9690 reclaim</t>
+          <t>₹3333 pullback</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>₹9265</t>
+          <t>₹3070</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>A- setup. Fresh box breakout to ATH 10,126, now pulling back. Enter 25% pilot on reclaim of 10D EMA 9,690. Add 50% above 10,126. Invalidate below 50D 9,265.</t>
+          <t>WAIT — extended late-stage (box 5+), weekly reversal -4.9%. Only on orderly pullback to 21D ~3,333 holding. Never chase above 3,600.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>ACUTAAS</t>
+          <t>RSI</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>₹3333 pullback</t>
+          <t>$29.69-30.00</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>₹3070</t>
+          <t>$29.24</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>WAIT — extended late-stage (box 5+), weekly reversal -4.9%. Only on orderly pullback to 21D ~3,333 holding. Never chase above 3,600.</t>
+          <t>US gaming. Pullback entry to Darvas trail. Skip on close below 29.24.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>RSI</t>
+          <t>STX</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>$29.69-30.00</t>
+          <t>$475-510</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>$29.24</t>
+          <t>$448</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>US gaming. Pullback entry to Darvas trail. Skip on close below 29.24.</t>
+          <t>US semis. B+ setup — RE-CHECK after global chip selloff before acting.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>STX</t>
+          <t>WAAREEENER</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>$475-510</t>
+          <t>₹3080-3120</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>$448</t>
+          <t>₹2960</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>US semis. B+ setup — RE-CHECK after global chip selloff before acting.</t>
+          <t>B- setup. Wait for ATH &gt;3800.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>WAAREEENER</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>₹3080-3120</t>
+          <t>₹1280-1320</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>₹2960</t>
+          <t>₹1177</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>B- setup. Wait for ATH &gt;3800.</t>
+          <t>C+ setup — WAIT. Extended. Only on pullback to 10W EMA ~1280. Remove if closes below 21W 1177.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>₹1280-1320</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>₹1177</t>
-        </is>
-      </c>
+          <t>NIFTY</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr"/>
+      <c r="C16" s="5" t="inlineStr"/>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>C+ setup — WAIT. Extended. Only on pullback to 10W EMA ~1280. Remove if closes below 21W 1177.</t>
+          <t>RULE FIRED 2026-08-14: price 24,202 lost 21D EMA (24,326) AND 10D EMA (24,374) AND 150D SMA (24,294) AND 200D SMA (24,714) — only above 50D (24,124). Do not deploy new swing longs beyond pilot size until 21D EMA reclaimed.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>NIFTY</t>
+          <t>NIFTY500</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr"/>
       <c r="C17" s="5" t="inlineStr"/>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>RULE FIRED 2026-08-14: price 24,202 lost 21D EMA (24,326) AND 10D EMA (24,374) AND 150D SMA (24,294) AND 200D SMA (24,714) — only above 50D (24,124). Do not deploy new swing longs beyond pilot size until 21D EMA reclaimed.</t>
+          <t>Weaker but not broken: price 23,508 below 10D EMA (23,591) only, still above 21D/50D/150D/200D. Broader-market gauge for mid/small-cap names (more relevant than Nifty50 for names like NETWEB). RS vs Nasdaq at 11 (bottom decile), falling.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>NIFTY500</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr"/>
       <c r="C18" s="5" t="inlineStr"/>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Weaker but not broken: price 23,508 below 10D EMA (23,591) only, still above 21D/50D/150D/200D. Broader-market gauge for mid/small-cap names (more relevant than Nifty50 for names like NETWEB). RS vs Nasdaq at 11 (bottom decile), falling.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="inlineStr"/>
-      <c r="C19" s="5" t="inlineStr"/>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
           <t>US regime gauge — chip selloff in progress, watch for follow-through distribution</t>
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Closed Trade Journal</t>
+        </is>
+      </c>
+    </row>
     <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>Closed Trade Journal</t>
-        </is>
-      </c>
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Avg Entry</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>Avg Exit</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>P&amp;L %</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>Hold Days</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr"/>
+      <c r="I21" s="4" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="4" t="inlineStr">
-        <is>
-          <t>Ticker</t>
-        </is>
-      </c>
-      <c r="B22" s="4" t="inlineStr">
-        <is>
-          <t>Result</t>
-        </is>
-      </c>
-      <c r="C22" s="4" t="inlineStr">
-        <is>
-          <t>Avg Entry</t>
-        </is>
-      </c>
-      <c r="D22" s="4" t="inlineStr">
-        <is>
-          <t>Avg Exit</t>
-        </is>
-      </c>
-      <c r="E22" s="4" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
-      </c>
-      <c r="F22" s="4" t="inlineStr">
-        <is>
-          <t>P&amp;L %</t>
-        </is>
-      </c>
-      <c r="G22" s="4" t="inlineStr">
-        <is>
-          <t>Hold Days</t>
-        </is>
-      </c>
-      <c r="H22" s="4" t="inlineStr"/>
-      <c r="I22" s="4" t="inlineStr"/>
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>SNDK</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>profit</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="n">
+        <v>903.13</v>
+      </c>
+      <c r="D22" s="5" t="n">
+        <v>1250.83</v>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>$113</t>
+        </is>
+      </c>
+      <c r="F22" s="21" t="n">
+        <v>37.7</v>
+      </c>
+      <c r="G22" s="5" t="n">
+        <v>35</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>SNDK</t>
+          <t>BSE.NS</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
@@ -4224,85 +4243,85 @@
         </is>
       </c>
       <c r="C23" s="5" t="n">
-        <v>903.13</v>
+        <v>3415.5</v>
       </c>
       <c r="D23" s="5" t="n">
-        <v>1250.83</v>
+        <v>3994.53</v>
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>$113</t>
+          <t>₹4,632</t>
         </is>
       </c>
       <c r="F23" s="21" t="n">
-        <v>37.7</v>
+        <v>17</v>
       </c>
       <c r="G23" s="5" t="n">
-        <v>35</v>
+        <v>48</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>BSE.NS</t>
+          <t>KRN</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>profit</t>
+          <t>loss</t>
         </is>
       </c>
       <c r="C24" s="5" t="n">
-        <v>3415.5</v>
+        <v>1310</v>
       </c>
       <c r="D24" s="5" t="n">
-        <v>3994.53</v>
+        <v>1197.27</v>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>₹4,632</t>
-        </is>
-      </c>
-      <c r="F24" s="21" t="n">
-        <v>17</v>
+          <t>₹-2,480</t>
+        </is>
+      </c>
+      <c r="F24" s="23" t="n">
+        <v>-8.6</v>
       </c>
       <c r="G24" s="5" t="n">
-        <v>48</v>
+        <v>9</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>KRN</t>
+          <t>CPRX</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>loss</t>
+          <t>profit</t>
         </is>
       </c>
       <c r="C25" s="5" t="n">
-        <v>1310</v>
+        <v>28.03</v>
       </c>
       <c r="D25" s="5" t="n">
-        <v>1197.27</v>
+        <v>31.14</v>
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>₹-2,480</t>
-        </is>
-      </c>
-      <c r="F25" s="23" t="n">
-        <v>-8.6</v>
+          <t>$21</t>
+        </is>
+      </c>
+      <c r="F25" s="21" t="n">
+        <v>10.4</v>
       </c>
       <c r="G25" s="5" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>CPRX</t>
+          <t>ATHERENERG</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
@@ -4311,123 +4330,93 @@
         </is>
       </c>
       <c r="C26" s="5" t="n">
-        <v>28.03</v>
+        <v>960.4</v>
       </c>
       <c r="D26" s="5" t="n">
-        <v>31.14</v>
+        <v>979.5</v>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>$21</t>
+          <t>₹134</t>
         </is>
       </c>
       <c r="F26" s="21" t="n">
-        <v>10.4</v>
+        <v>2</v>
       </c>
       <c r="G26" s="5" t="n">
-        <v>14</v>
+        <v>37</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>ATHERENERG</t>
+          <t>LRCX</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>profit</t>
+          <t>scratch</t>
         </is>
       </c>
       <c r="C27" s="5" t="n">
-        <v>960.4</v>
+        <v>346.09</v>
       </c>
       <c r="D27" s="5" t="n">
-        <v>979.5</v>
+        <v>346</v>
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>₹134</t>
-        </is>
-      </c>
-      <c r="F27" s="21" t="n">
-        <v>2</v>
+          <t>$-0</t>
+        </is>
+      </c>
+      <c r="F27" s="23" t="n">
+        <v>-0.03</v>
       </c>
       <c r="G27" s="5" t="n">
-        <v>37</v>
+        <v>27</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>LRCX</t>
+          <t>DATAPATTNS</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>scratch</t>
+          <t>loss</t>
         </is>
       </c>
       <c r="C28" s="5" t="n">
-        <v>346.09</v>
+        <v>4805</v>
       </c>
       <c r="D28" s="5" t="n">
-        <v>346</v>
+        <v>4400</v>
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>$-0</t>
+          <t>₹-4,050</t>
         </is>
       </c>
       <c r="F28" s="23" t="n">
-        <v>-0.03</v>
-      </c>
-      <c r="G28" s="5" t="n">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="5" t="inlineStr">
-        <is>
-          <t>DATAPATTNS</t>
-        </is>
-      </c>
-      <c r="B29" s="5" t="inlineStr">
-        <is>
-          <t>loss</t>
-        </is>
-      </c>
-      <c r="C29" s="5" t="n">
-        <v>4805</v>
-      </c>
-      <c r="D29" s="5" t="n">
-        <v>4400</v>
-      </c>
-      <c r="E29" s="5" t="inlineStr">
-        <is>
-          <t>₹-4,050</t>
-        </is>
-      </c>
-      <c r="F29" s="23" t="n">
         <v>-8.4</v>
       </c>
-      <c r="G29" s="5" t="n"/>
+      <c r="G28" s="5" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="14">
-    <mergeCell ref="D19:I19"/>
-    <mergeCell ref="A7:I7"/>
+  <mergeCells count="13">
     <mergeCell ref="D11:I11"/>
+    <mergeCell ref="D10:I10"/>
     <mergeCell ref="D13:I13"/>
+    <mergeCell ref="A5:I5"/>
     <mergeCell ref="D14:I14"/>
     <mergeCell ref="D18:I18"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="D17:I17"/>
-    <mergeCell ref="A9:I9"/>
+    <mergeCell ref="A8:I8"/>
     <mergeCell ref="D12:I12"/>
     <mergeCell ref="D16:I16"/>
-    <mergeCell ref="A4:I4"/>
-    <mergeCell ref="A21:I21"/>
+    <mergeCell ref="A20:I20"/>
     <mergeCell ref="D15:I15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4566,7 +4555,7 @@
         <f>(H3-G3)*F3</f>
         <v/>
       </c>
-      <c r="K3" s="26">
+      <c r="K3" s="25">
         <f>IF(G3&gt;0,(H3-G3)/G3,0)</f>
         <v/>
       </c>
@@ -4615,7 +4604,7 @@
         <f>(H4-G4)*F4</f>
         <v/>
       </c>
-      <c r="K4" s="26">
+      <c r="K4" s="25">
         <f>IF(G4&gt;0,(H4-G4)/G4,0)</f>
         <v/>
       </c>
@@ -4664,7 +4653,7 @@
         <f>(H5-G5)*F5</f>
         <v/>
       </c>
-      <c r="K5" s="26">
+      <c r="K5" s="25">
         <f>IF(G5&gt;0,(H5-G5)/G5,0)</f>
         <v/>
       </c>
@@ -4713,7 +4702,7 @@
         <f>(H6-G6)*F6</f>
         <v/>
       </c>
-      <c r="K6" s="26">
+      <c r="K6" s="25">
         <f>IF(G6&gt;0,(H6-G6)/G6,0)</f>
         <v/>
       </c>
@@ -4762,7 +4751,7 @@
         <f>(H7-G7)*F7</f>
         <v/>
       </c>
-      <c r="K7" s="26">
+      <c r="K7" s="25">
         <f>IF(G7&gt;0,(H7-G7)/G7,0)</f>
         <v/>
       </c>
@@ -4811,7 +4800,7 @@
         <f>(H8-G8)*F8</f>
         <v/>
       </c>
-      <c r="K8" s="26">
+      <c r="K8" s="25">
         <f>IF(G8&gt;0,(H8-G8)/G8,0)</f>
         <v/>
       </c>
@@ -4860,7 +4849,7 @@
         <f>(H9-G9)*F9</f>
         <v/>
       </c>
-      <c r="K9" s="26">
+      <c r="K9" s="25">
         <f>IF(G9&gt;0,(H9-G9)/G9,0)</f>
         <v/>
       </c>
@@ -5125,7 +5114,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="27" t="inlineStr">
+      <c r="A1" s="26" t="inlineStr">
         <is>
           <t>POSITION SIZING &amp; R:R CALCULATOR</t>
         </is>
@@ -5146,42 +5135,42 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="28" t="inlineStr">
+      <c r="A5" s="27" t="inlineStr">
         <is>
           <t>Entry price</t>
         </is>
       </c>
-      <c r="B5" s="29" t="n">
+      <c r="B5" s="28" t="n">
         <v>100</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="28" t="inlineStr">
+      <c r="A6" s="27" t="inlineStr">
         <is>
           <t>Stop loss</t>
         </is>
       </c>
-      <c r="B6" s="29" t="n">
+      <c r="B6" s="28" t="n">
         <v>92</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="28" t="inlineStr">
+      <c r="A7" s="27" t="inlineStr">
         <is>
           <t>Account / sleeve ₹</t>
         </is>
       </c>
-      <c r="B7" s="30" t="n">
+      <c r="B7" s="29" t="n">
         <v>263453</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="28" t="inlineStr">
+      <c r="A8" s="27" t="inlineStr">
         <is>
           <t>Risk budget %</t>
         </is>
       </c>
-      <c r="B8" s="31" t="n">
+      <c r="B8" s="30" t="n">
         <v>2</v>
       </c>
     </row>
@@ -5193,67 +5182,67 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="28" t="inlineStr">
+      <c r="A11" s="27" t="inlineStr">
         <is>
           <t>Risk per share</t>
         </is>
       </c>
-      <c r="B11" s="32">
+      <c r="B11" s="31">
         <f>B5-B6</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="28" t="inlineStr">
+      <c r="A12" s="27" t="inlineStr">
         <is>
           <t>Risk % of entry</t>
         </is>
       </c>
-      <c r="B12" s="33">
+      <c r="B12" s="32">
         <f>(B5-B6)/B5</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="28" t="inlineStr">
+      <c r="A13" s="27" t="inlineStr">
         <is>
           <t>Max ₹ at risk</t>
         </is>
       </c>
-      <c r="B13" s="34">
+      <c r="B13" s="33">
         <f>B7*B8/100</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="28" t="inlineStr">
+      <c r="A14" s="27" t="inlineStr">
         <is>
           <t>Max shares</t>
         </is>
       </c>
-      <c r="B14" s="34">
+      <c r="B14" s="33">
         <f>IF(B11&gt;0,FLOOR(B13/B11,1),0)</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="28" t="inlineStr">
+      <c r="A15" s="27" t="inlineStr">
         <is>
           <t>Capital required</t>
         </is>
       </c>
-      <c r="B15" s="34">
+      <c r="B15" s="33">
         <f>B14*B5</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="28" t="inlineStr">
+      <c r="A16" s="27" t="inlineStr">
         <is>
           <t>% of sleeve deployed</t>
         </is>
       </c>
-      <c r="B16" s="35">
+      <c r="B16" s="34">
         <f>IF(B7&gt;0,B15/B7,0)</f>
         <v/>
       </c>
@@ -5266,34 +5255,34 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="28" t="inlineStr">
+      <c r="A19" s="27" t="inlineStr">
         <is>
           <t>T1 pilot (25%)</t>
         </is>
       </c>
-      <c r="B19" s="34">
+      <c r="B19" s="33">
         <f>FLOOR(B14*0.25,1)</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="28" t="inlineStr">
+      <c r="A20" s="27" t="inlineStr">
         <is>
           <t>T2 core (50%)</t>
         </is>
       </c>
-      <c r="B20" s="34">
+      <c r="B20" s="33">
         <f>FLOOR(B14*0.5,1)</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="28" t="inlineStr">
+      <c r="A21" s="27" t="inlineStr">
         <is>
           <t>T3 final (25%)</t>
         </is>
       </c>
-      <c r="B21" s="34">
+      <c r="B21" s="33">
         <f>B14-B19-B20</f>
         <v/>
       </c>
@@ -5306,163 +5295,163 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="36" t="inlineStr">
+      <c r="A24" s="35" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="B24" s="36" t="inlineStr">
+      <c r="B24" s="35" t="inlineStr">
         <is>
           <t>Price</t>
         </is>
       </c>
-      <c r="C24" s="36" t="inlineStr">
+      <c r="C24" s="35" t="inlineStr">
         <is>
           <t>% of position</t>
         </is>
       </c>
-      <c r="D24" s="36" t="inlineStr">
+      <c r="D24" s="35" t="inlineStr">
         <is>
           <t>R:R</t>
         </is>
       </c>
-      <c r="E24" s="36" t="inlineStr">
+      <c r="E24" s="35" t="inlineStr">
         <is>
           <t>Reward %</t>
         </is>
       </c>
-      <c r="F24" s="36" t="inlineStr">
+      <c r="F24" s="35" t="inlineStr">
         <is>
           <t>P&amp;L ₹ (at max shares)</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="28" t="inlineStr">
+      <c r="A25" s="27" t="inlineStr">
         <is>
           <t>T1</t>
         </is>
       </c>
-      <c r="B25" s="29" t="n">
+      <c r="B25" s="28" t="n">
         <v>110</v>
       </c>
-      <c r="C25" s="37" t="n">
+      <c r="C25" s="36" t="n">
         <v>33</v>
       </c>
-      <c r="D25" s="38">
+      <c r="D25" s="37">
         <f>IF($B$5-$B$6&gt;0,(B25-$B$5)/($B$5-$B$6),0)</f>
         <v/>
       </c>
-      <c r="E25" s="35">
+      <c r="E25" s="34">
         <f>(B25-$B$5)/$B$5</f>
         <v/>
       </c>
-      <c r="F25" s="34">
+      <c r="F25" s="33">
         <f>(B25-$B$5)*FLOOR($B$14*C25/100,1)</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="28" t="inlineStr">
+      <c r="A26" s="27" t="inlineStr">
         <is>
           <t>T2</t>
         </is>
       </c>
-      <c r="B26" s="29" t="n">
+      <c r="B26" s="28" t="n">
         <v>120</v>
       </c>
-      <c r="C26" s="37" t="n">
+      <c r="C26" s="36" t="n">
         <v>33</v>
       </c>
-      <c r="D26" s="38">
+      <c r="D26" s="37">
         <f>IF($B$5-$B$6&gt;0,(B26-$B$5)/($B$5-$B$6),0)</f>
         <v/>
       </c>
-      <c r="E26" s="35">
+      <c r="E26" s="34">
         <f>(B26-$B$5)/$B$5</f>
         <v/>
       </c>
-      <c r="F26" s="34">
+      <c r="F26" s="33">
         <f>(B26-$B$5)*FLOOR($B$14*C26/100,1)</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="28" t="inlineStr">
+      <c r="A27" s="27" t="inlineStr">
         <is>
           <t>T3</t>
         </is>
       </c>
-      <c r="B27" s="29" t="n">
+      <c r="B27" s="28" t="n">
         <v>135</v>
       </c>
-      <c r="C27" s="37" t="n">
+      <c r="C27" s="36" t="n">
         <v>34</v>
       </c>
-      <c r="D27" s="38">
+      <c r="D27" s="37">
         <f>IF($B$5-$B$6&gt;0,(B27-$B$5)/($B$5-$B$6),0)</f>
         <v/>
       </c>
-      <c r="E27" s="35">
+      <c r="E27" s="34">
         <f>(B27-$B$5)/$B$5</f>
         <v/>
       </c>
-      <c r="F27" s="34">
+      <c r="F27" s="33">
         <f>(B27-$B$5)*FLOOR($B$14*C27/100,1)</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="39" t="inlineStr">
+      <c r="A28" s="38" t="inlineStr">
         <is>
           <t>Weighted avg R:R</t>
         </is>
       </c>
-      <c r="D28" s="38">
+      <c r="D28" s="37">
         <f>IF(SUM(C25:C27)&gt;0,SUMPRODUCT(D25:D27,C25:C27)/SUM(C25:C27),0)</f>
         <v/>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="39" t="inlineStr">
+      <c r="A29" s="38" t="inlineStr">
         <is>
           <t>Avg exit price</t>
         </is>
       </c>
-      <c r="B29" s="32">
+      <c r="B29" s="31">
         <f>IF(SUM(C25:C27)&gt;0,SUMPRODUCT(B25:B27,C25:C27)/SUM(C25:C27),0)</f>
         <v/>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="39" t="inlineStr">
+      <c r="A30" s="38" t="inlineStr">
         <is>
           <t>Full-run P&amp;L ₹</t>
         </is>
       </c>
-      <c r="B30" s="34">
+      <c r="B30" s="33">
         <f>SUM(F25:F27)</f>
         <v/>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="39" t="inlineStr">
+      <c r="A31" s="38" t="inlineStr">
         <is>
           <t>Payoff ratio (win/loss)</t>
         </is>
       </c>
-      <c r="B31" s="38">
+      <c r="B31" s="37">
         <f>IF(B13&gt;0,B30/B13,0)</f>
         <v/>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="39" t="inlineStr">
+      <c r="A32" s="38" t="inlineStr">
         <is>
           <t>Break-even win rate</t>
         </is>
       </c>
-      <c r="B32" s="35">
+      <c r="B32" s="34">
         <f>IF(B31&gt;0,1/(1+B31),0)</f>
         <v/>
       </c>
@@ -5590,7 +5579,7 @@
       <c r="I3" s="21" t="n">
         <v>30.59031517163864</v>
       </c>
-      <c r="J3" s="40" t="inlineStr">
+      <c r="J3" s="39" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -5635,7 +5624,7 @@
       <c r="I5" s="23" t="n">
         <v>-23.05421294278932</v>
       </c>
-      <c r="J5" s="41" t="inlineStr">
+      <c r="J5" s="40" t="inlineStr">
         <is>
           <t>HOLD_FOR_TLH</t>
         </is>
@@ -5672,7 +5661,7 @@
       <c r="G7" s="6" t="n"/>
       <c r="H7" s="6" t="n"/>
       <c r="I7" s="5" t="n"/>
-      <c r="J7" s="42" t="inlineStr">
+      <c r="J7" s="41" t="inlineStr">
         <is>
           <t>SOLD</t>
         </is>

</xml_diff>

<commit_message>
Close NETWEB — stopped out on Nifty distribution day
Exit ~₹5,085 (SL-M trigger, estimated — exact fill/date pending contract
note confirmation). Loss ₹1,578 (-4.92%, -1.0R), matching the planned
tactical stop exactly. Regime-gating call proved out: the Nifty 50 21D
EMA break flagged the prior day turned into the broad selloff that
stopped this out. Growth sleeve back to fully flat, cash 1,198,422.

Added closed_swing_positions journal to father_portfolio.yaml and a
matching "Closed Swing/Growth Journal" section to the Father tab in
portfolio_tracker.py.

https://claude.ai/code/session_01HhF36NsLiVFyxhhXe4S24m
</commit_message>
<xml_diff>
--- a/examples/swing_monitor/Portfolio_Tracker.xlsx
+++ b/examples/swing_monitor/Portfolio_Tracker.xlsx
@@ -575,7 +575,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-18 09:09  |  USD/INR 95.0  |  prices: override file (2026-08-12T10:29:00+00:00), yfinance off</t>
+          <t>Generated 2026-08-19 17:05  |  USD/INR 95.0  |  prices: override file (2026-08-12T10:29:00+00:00), yfinance off</t>
         </is>
       </c>
     </row>
@@ -5400,7 +5400,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J21"/>
+  <dimension ref="A1:J23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5627,7 +5627,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Source: Colgate-Palmolive sale proceeds  |  Pool: ₹1,200,000  |  Risk/trade: 1%  |  Deployed: ₹32,088  |  Cash remaining: ₹1,167,912</t>
+          <t>Source: Colgate-Palmolive sale proceeds  |  Pool: ₹1,200,000  |  Risk/trade: 1%  |  Deployed: ₹0  |  Cash remaining: ₹1,198,422</t>
         </is>
       </c>
     </row>
@@ -5639,129 +5639,115 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>Ticker</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>Qty</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>Entry</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>LTP</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>Stop</t>
-        </is>
-      </c>
-      <c r="F15" s="4" t="inlineStr">
-        <is>
-          <t>Next Target</t>
-        </is>
-      </c>
-      <c r="G15" s="4" t="inlineStr">
-        <is>
-          <t>P&amp;L %</t>
-        </is>
-      </c>
-      <c r="H15" s="4" t="inlineStr">
-        <is>
-          <t>Risk ₹</t>
-        </is>
-      </c>
-      <c r="I15" s="4" t="inlineStr">
-        <is>
-          <t>Src</t>
-        </is>
-      </c>
-      <c r="J15" s="4" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>NETWEB</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="C16" s="13" t="n">
-        <v>5348</v>
-      </c>
-      <c r="D16" s="13" t="n">
-        <v>5314.05</v>
-      </c>
-      <c r="E16" s="13" t="n">
-        <v>5085</v>
-      </c>
-      <c r="F16" s="13" t="n">
-        <v>5800</v>
-      </c>
-      <c r="G16" s="23" t="n">
-        <v>-0.6348167539267036</v>
-      </c>
-      <c r="H16" s="6" t="n">
-        <v>1578</v>
-      </c>
-      <c r="I16" s="5" t="inlineStr">
-        <is>
-          <t>override</t>
-        </is>
-      </c>
-      <c r="J16" s="5" t="inlineStr">
-        <is>
-          <t>open</t>
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>No active swing/growth positions.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>↳ Plan: PILOT 6sh FILLED @5348 2026-08-14 via HDFC Securities. CORE 12sh GATED: only after Nifty 50 reclaims 21D EMA (24,326) and ideally 150D SMA (24,294), OR a recognized O'Neil follow-through day. FINAL 6sh at/after T1 (5800), pullback to 10D EMA holds. Stop to breakeven after Core fills; trail 10D/21D EMA after Final.</t>
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Planned Trades (redeployment of sale proceeds)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>↳ Notes: Reverse-pyramid / 25-50-25 tranche plan. Working stop 5,085 (SL-M, day-1-low based) tighter than structural 4,825 — appropriate given regime caution. Risk ₹1,578 (0.13% of growth_sleeve). Core/Final regime-gated on Nifty 50 21D EMA reclaim.</t>
+          <t>None yet — ~₹50L expected free after GILLETTE + COLPAL exits. Plan before redeploying.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Planned Trades (redeployment of sale proceeds)</t>
+          <t>Closed Swing/Growth Journal</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>None yet — ~₹50L expected free after GILLETTE + COLPAL exits. Plan before redeploying.</t>
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Avg Entry</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>Avg Exit</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>P&amp;L %</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr"/>
+      <c r="I21" s="4" t="inlineStr"/>
+      <c r="J21" s="4" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>NETWEB</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>loss</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="n">
+        <v>5348</v>
+      </c>
+      <c r="D22" s="5" t="n">
+        <v>5085</v>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>₹-1,578</t>
+        </is>
+      </c>
+      <c r="F22" s="23" t="n">
+        <v>-4.92</v>
+      </c>
+      <c r="G22" s="19" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>↳ Stopped out via SL-M ~5,085 on a Nifty distribution day — stock down ~5% intraday from prior close on market-wide instability, not company-specific news. Exit price is an ESTIMATE (SL-M trigger level) — CONFIRM exact fill + exact date from the HDFC Securities contract note. Textbook outcome of the regime-gating call: the Nifty 50 21D EMA loss flagged the day before turned into exactly the kind of broad selloff that stops out pilot positions. Working stop (day-1-low based, tighter than the 4,825 structural level) did its job — loss capped at planned 0.13% of sleeve, no damage beyond the plan.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="9">
     <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A23:J23"/>
     <mergeCell ref="A14:J14"/>
     <mergeCell ref="A17:J17"/>
-    <mergeCell ref="A18:J18"/>
     <mergeCell ref="B8:J8"/>
     <mergeCell ref="A20:J20"/>
     <mergeCell ref="B4:J4"/>

</xml_diff>

<commit_message>
Log Dorian LPG (LPG) as planned trade — Vishesh's own INDmoney/Alpaca account
$1,000 available, 1% max risk ($10), stop at breakout pivot ($48.00) per
explicit choice — 2.8% stop distance. 7 shares (~$345.73, ~35% of
account). R:R to consensus PT ($55) is 4.0:1, reflecting the tight stop.

Flagged explicitly as event-driven (Strait of Hormuz disruption spiking
VLGC freight rates), not structural growth like NETWEB — earnings beat
and record TCE/day are catalyst-driven, and a holding ceasefire is the
single biggest risk to the thesis, separate from and faster-moving than
what the chart alone shows. Corrected an earlier chart-reading error:
orange line is TTM diluted EPS, not the 150D SMA.

https://claude.ai/code/session_01HhF36NsLiVFyxhhXe4S24m
</commit_message>
<xml_diff>
--- a/examples/swing_monitor/Portfolio_Tracker.xlsx
+++ b/examples/swing_monitor/Portfolio_Tracker.xlsx
@@ -105,6 +105,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00FEF3C7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00FEF9C3"/>
       </patternFill>
     </fill>
@@ -116,11 +121,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00DCFCE7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FEF3C7"/>
       </patternFill>
     </fill>
     <fill>
@@ -146,7 +146,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -174,22 +174,23 @@
     <xf numFmtId="3" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="169" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -575,7 +576,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-19 17:05  |  USD/INR 95.0  |  prices: override file (2026-08-12T10:29:00+00:00), yfinance off</t>
+          <t>Generated 2026-08-19 17:48  |  USD/INR 95.0  |  prices: override file (2026-08-12T10:29:00+00:00), yfinance off</t>
         </is>
       </c>
     </row>
@@ -3833,7 +3834,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I27"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3869,357 +3870,381 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>No planned positions.</t>
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Plan Qty</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Pilot Entry</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>LTP</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Pivot</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>Dist to Buy Zone</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>Risk ₹ (full)</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>Src</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="25" t="inlineStr">
+        <is>
+          <t>LPG</t>
+        </is>
+      </c>
+      <c r="B6" s="25" t="n">
+        <v>7</v>
+      </c>
+      <c r="C6" s="25" t="n">
+        <v>49.39</v>
+      </c>
+      <c r="D6" s="25" t="n">
+        <v>49.39</v>
+      </c>
+      <c r="E6" s="25" t="n">
+        <v>48</v>
+      </c>
+      <c r="F6" s="25" t="n">
+        <v>48</v>
+      </c>
+      <c r="G6" s="25" t="inlineStr">
+        <is>
+          <t>IN ZONE</t>
+        </is>
+      </c>
+      <c r="H6" s="25" t="n">
+        <v>9.730000000000004</v>
+      </c>
+      <c r="I6" s="25" t="inlineStr">
+        <is>
+          <t>override</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>↳ LPG: Single clean entry ~7sh (not tranched, small account). Stop AT breakout pivot $48 per explicit choice — tight 2.8% stop, expect higher stop-out frequency than a wider stop in exchange for hard-capped $10 loss. Watch ceasefire news as a fundamental override signal independent of price action.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Watchlist / Planned Entries</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>Trigger</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>Stop</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr"/>
-      <c r="F8" s="4" t="inlineStr"/>
-      <c r="G8" s="4" t="inlineStr"/>
-      <c r="H8" s="4" t="inlineStr"/>
-      <c r="I8" s="4" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>POLYCAB</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>₹9690 reclaim</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>₹9265</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>A- setup. Fresh box breakout to ATH 10,126, now pulling back. Enter 25% pilot on reclaim of 10D EMA 9,690. Add 50% above 10,126. Invalidate below 50D 9,265.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>ACUTAAS</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>₹3333 pullback</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>₹3070</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>WAIT — extended late-stage (box 5+), weekly reversal -4.9%. Only on orderly pullback to 21D ~3,333 holding. Never chase above 3,600.</t>
-        </is>
-      </c>
+      <c r="E10" s="4" t="inlineStr"/>
+      <c r="F10" s="4" t="inlineStr"/>
+      <c r="G10" s="4" t="inlineStr"/>
+      <c r="H10" s="4" t="inlineStr"/>
+      <c r="I10" s="4" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>RSI</t>
+          <t>POLYCAB</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>$29.69-30.00</t>
+          <t>₹9690 reclaim</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>$29.24</t>
+          <t>₹9265</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>US gaming. Pullback entry to Darvas trail. Skip on close below 29.24.</t>
+          <t>A- setup. Fresh box breakout to ATH 10,126, now pulling back. Enter 25% pilot on reclaim of 10D EMA 9,690. Add 50% above 10,126. Invalidate below 50D 9,265.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>STX</t>
+          <t>ACUTAAS</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>$475-510</t>
+          <t>₹3333 pullback</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>$448</t>
+          <t>₹3070</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>US semis. B+ setup — RE-CHECK after global chip selloff before acting.</t>
+          <t>WAIT — extended late-stage (box 5+), weekly reversal -4.9%. Only on orderly pullback to 21D ~3,333 holding. Never chase above 3,600.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>WAAREEENER</t>
+          <t>RSI</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>₹3080-3120</t>
+          <t>$29.69-30.00</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>₹2960</t>
+          <t>$29.24</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>B- setup. Wait for ATH &gt;3800.</t>
+          <t>US gaming. Pullback entry to Darvas trail. Skip on close below 29.24.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>STX</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>₹1280-1320</t>
+          <t>$475-510</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>₹1177</t>
+          <t>$448</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>C+ setup — WAIT. Extended. Only on pullback to 10W EMA ~1280. Remove if closes below 21W 1177.</t>
+          <t>US semis. B+ setup — RE-CHECK after global chip selloff before acting.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>NIFTY</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr"/>
-      <c r="C15" s="5" t="inlineStr"/>
+          <t>WAAREEENER</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>₹3080-3120</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>₹2960</t>
+        </is>
+      </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>RULE FIRED 2026-08-14: price 24,202 lost 21D EMA (24,326) AND 10D EMA (24,374) AND 150D SMA (24,294) AND 200D SMA (24,714) — only above 50D (24,124). Do not deploy new swing longs beyond pilot size until 21D EMA reclaimed.</t>
+          <t>B- setup. Wait for ATH &gt;3800.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>NIFTY500</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr"/>
-      <c r="C16" s="5" t="inlineStr"/>
+          <t>LAURUSLABS</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>₹1280-1320</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>₹1177</t>
+        </is>
+      </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Weaker but not broken: price 23,508 below 10D EMA (23,591) only, still above 21D/50D/150D/200D. Broader-market gauge for mid/small-cap names (more relevant than Nifty50 for names like NETWEB). RS vs Nasdaq at 11 (bottom decile), falling.</t>
+          <t>C+ setup — WAIT. Extended. Only on pullback to 10W EMA ~1280. Remove if closes below 21W 1177.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>NIFTY</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr"/>
       <c r="C17" s="5" t="inlineStr"/>
       <c r="D17" s="2" t="inlineStr">
         <is>
+          <t>RULE FIRED 2026-08-14: price 24,202 lost 21D EMA (24,326) AND 10D EMA (24,374) AND 150D SMA (24,294) AND 200D SMA (24,714) — only above 50D (24,124). Do not deploy new swing longs beyond pilot size until 21D EMA reclaimed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>NIFTY500</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr"/>
+      <c r="C18" s="5" t="inlineStr"/>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Weaker but not broken: price 23,508 below 10D EMA (23,591) only, still above 21D/50D/150D/200D. Broader-market gauge for mid/small-cap names (more relevant than Nifty50 for names like NETWEB). RS vs Nasdaq at 11 (bottom decile), falling.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr"/>
+      <c r="C19" s="5" t="inlineStr"/>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
           <t>US regime gauge — chip selloff in progress, watch for follow-through distribution</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>Closed Trade Journal</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B20" s="4" t="inlineStr">
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>Result</t>
         </is>
       </c>
-      <c r="C20" s="4" t="inlineStr">
+      <c r="C22" s="4" t="inlineStr">
         <is>
           <t>Avg Entry</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
+      <c r="D22" s="4" t="inlineStr">
         <is>
           <t>Avg Exit</t>
         </is>
       </c>
-      <c r="E20" s="4" t="inlineStr">
+      <c r="E22" s="4" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
       </c>
-      <c r="F20" s="4" t="inlineStr">
+      <c r="F22" s="4" t="inlineStr">
         <is>
           <t>P&amp;L %</t>
         </is>
       </c>
-      <c r="G20" s="4" t="inlineStr">
+      <c r="G22" s="4" t="inlineStr">
         <is>
           <t>Hold Days</t>
         </is>
       </c>
-      <c r="H20" s="4" t="inlineStr"/>
-      <c r="I20" s="4" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="5" t="inlineStr">
-        <is>
-          <t>SNDK</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="inlineStr">
-        <is>
-          <t>profit</t>
-        </is>
-      </c>
-      <c r="C21" s="5" t="n">
-        <v>903.13</v>
-      </c>
-      <c r="D21" s="5" t="n">
-        <v>1250.83</v>
-      </c>
-      <c r="E21" s="5" t="inlineStr">
-        <is>
-          <t>$113</t>
-        </is>
-      </c>
-      <c r="F21" s="21" t="n">
-        <v>37.7</v>
-      </c>
-      <c r="G21" s="5" t="n">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="5" t="inlineStr">
-        <is>
-          <t>BSE.NS</t>
-        </is>
-      </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>profit</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="n">
-        <v>3415.5</v>
-      </c>
-      <c r="D22" s="5" t="n">
-        <v>3994.53</v>
-      </c>
-      <c r="E22" s="5" t="inlineStr">
-        <is>
-          <t>₹4,632</t>
-        </is>
-      </c>
-      <c r="F22" s="21" t="n">
-        <v>17</v>
-      </c>
-      <c r="G22" s="5" t="n">
-        <v>48</v>
-      </c>
+      <c r="H22" s="4" t="inlineStr"/>
+      <c r="I22" s="4" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>KRN</t>
+          <t>SNDK</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>loss</t>
+          <t>profit</t>
         </is>
       </c>
       <c r="C23" s="5" t="n">
-        <v>1310</v>
+        <v>903.13</v>
       </c>
       <c r="D23" s="5" t="n">
-        <v>1197.27</v>
+        <v>1250.83</v>
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>₹-2,480</t>
-        </is>
-      </c>
-      <c r="F23" s="23" t="n">
-        <v>-8.6</v>
+          <t>$113</t>
+        </is>
+      </c>
+      <c r="F23" s="21" t="n">
+        <v>37.7</v>
       </c>
       <c r="G23" s="5" t="n">
-        <v>9</v>
+        <v>35</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>CPRX</t>
+          <t>BSE.NS</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
@@ -4228,122 +4253,181 @@
         </is>
       </c>
       <c r="C24" s="5" t="n">
-        <v>28.03</v>
+        <v>3415.5</v>
       </c>
       <c r="D24" s="5" t="n">
-        <v>31.14</v>
+        <v>3994.53</v>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>$21</t>
+          <t>₹4,632</t>
         </is>
       </c>
       <c r="F24" s="21" t="n">
-        <v>10.4</v>
+        <v>17</v>
       </c>
       <c r="G24" s="5" t="n">
-        <v>14</v>
+        <v>48</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>ATHERENERG</t>
+          <t>KRN</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>profit</t>
+          <t>loss</t>
         </is>
       </c>
       <c r="C25" s="5" t="n">
-        <v>960.4</v>
+        <v>1310</v>
       </c>
       <c r="D25" s="5" t="n">
-        <v>979.5</v>
+        <v>1197.27</v>
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>₹134</t>
-        </is>
-      </c>
-      <c r="F25" s="21" t="n">
-        <v>2</v>
+          <t>₹-2,480</t>
+        </is>
+      </c>
+      <c r="F25" s="23" t="n">
+        <v>-8.6</v>
       </c>
       <c r="G25" s="5" t="n">
-        <v>37</v>
+        <v>9</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>LRCX</t>
+          <t>CPRX</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>scratch</t>
+          <t>profit</t>
         </is>
       </c>
       <c r="C26" s="5" t="n">
-        <v>346.09</v>
+        <v>28.03</v>
       </c>
       <c r="D26" s="5" t="n">
-        <v>346</v>
+        <v>31.14</v>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>$-0</t>
-        </is>
-      </c>
-      <c r="F26" s="23" t="n">
-        <v>-0.03</v>
+          <t>$21</t>
+        </is>
+      </c>
+      <c r="F26" s="21" t="n">
+        <v>10.4</v>
       </c>
       <c r="G26" s="5" t="n">
-        <v>27</v>
+        <v>14</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
+          <t>ATHERENERG</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>profit</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="n">
+        <v>960.4</v>
+      </c>
+      <c r="D27" s="5" t="n">
+        <v>979.5</v>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>₹134</t>
+        </is>
+      </c>
+      <c r="F27" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="G27" s="5" t="n">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>LRCX</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>scratch</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="n">
+        <v>346.09</v>
+      </c>
+      <c r="D28" s="5" t="n">
+        <v>346</v>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>$-0</t>
+        </is>
+      </c>
+      <c r="F28" s="23" t="n">
+        <v>-0.03</v>
+      </c>
+      <c r="G28" s="5" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
           <t>DATAPATTNS</t>
         </is>
       </c>
-      <c r="B27" s="5" t="inlineStr">
+      <c r="B29" s="5" t="inlineStr">
         <is>
           <t>loss</t>
         </is>
       </c>
-      <c r="C27" s="5" t="n">
+      <c r="C29" s="5" t="n">
         <v>4805</v>
       </c>
-      <c r="D27" s="5" t="n">
+      <c r="D29" s="5" t="n">
         <v>4400</v>
       </c>
-      <c r="E27" s="5" t="inlineStr">
+      <c r="E29" s="5" t="inlineStr">
         <is>
           <t>₹-4,050</t>
         </is>
       </c>
-      <c r="F27" s="23" t="n">
+      <c r="F29" s="23" t="n">
         <v>-8.4</v>
       </c>
-      <c r="G27" s="5" t="n"/>
+      <c r="G29" s="5" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="14">
+    <mergeCell ref="D19:I19"/>
     <mergeCell ref="A7:I7"/>
     <mergeCell ref="D11:I11"/>
-    <mergeCell ref="D10:I10"/>
-    <mergeCell ref="A19:I19"/>
     <mergeCell ref="D13:I13"/>
     <mergeCell ref="D14:I14"/>
+    <mergeCell ref="D18:I18"/>
     <mergeCell ref="A1:I1"/>
-    <mergeCell ref="D9:I9"/>
     <mergeCell ref="D17:I17"/>
+    <mergeCell ref="A9:I9"/>
     <mergeCell ref="D12:I12"/>
     <mergeCell ref="D16:I16"/>
     <mergeCell ref="A4:I4"/>
+    <mergeCell ref="A21:I21"/>
     <mergeCell ref="D15:I15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4482,7 +4566,7 @@
         <f>(H3-G3)*F3</f>
         <v/>
       </c>
-      <c r="K3" s="25">
+      <c r="K3" s="26">
         <f>IF(G3&gt;0,(H3-G3)/G3,0)</f>
         <v/>
       </c>
@@ -4531,7 +4615,7 @@
         <f>(H4-G4)*F4</f>
         <v/>
       </c>
-      <c r="K4" s="25">
+      <c r="K4" s="26">
         <f>IF(G4&gt;0,(H4-G4)/G4,0)</f>
         <v/>
       </c>
@@ -4580,7 +4664,7 @@
         <f>(H5-G5)*F5</f>
         <v/>
       </c>
-      <c r="K5" s="25">
+      <c r="K5" s="26">
         <f>IF(G5&gt;0,(H5-G5)/G5,0)</f>
         <v/>
       </c>
@@ -4629,7 +4713,7 @@
         <f>(H6-G6)*F6</f>
         <v/>
       </c>
-      <c r="K6" s="25">
+      <c r="K6" s="26">
         <f>IF(G6&gt;0,(H6-G6)/G6,0)</f>
         <v/>
       </c>
@@ -4678,7 +4762,7 @@
         <f>(H7-G7)*F7</f>
         <v/>
       </c>
-      <c r="K7" s="25">
+      <c r="K7" s="26">
         <f>IF(G7&gt;0,(H7-G7)/G7,0)</f>
         <v/>
       </c>
@@ -4727,7 +4811,7 @@
         <f>(H8-G8)*F8</f>
         <v/>
       </c>
-      <c r="K8" s="25">
+      <c r="K8" s="26">
         <f>IF(G8&gt;0,(H8-G8)/G8,0)</f>
         <v/>
       </c>
@@ -4776,7 +4860,7 @@
         <f>(H9-G9)*F9</f>
         <v/>
       </c>
-      <c r="K9" s="25">
+      <c r="K9" s="26">
         <f>IF(G9&gt;0,(H9-G9)/G9,0)</f>
         <v/>
       </c>
@@ -5041,7 +5125,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="26" t="inlineStr">
+      <c r="A1" s="27" t="inlineStr">
         <is>
           <t>POSITION SIZING &amp; R:R CALCULATOR</t>
         </is>
@@ -5062,42 +5146,42 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="27" t="inlineStr">
+      <c r="A5" s="28" t="inlineStr">
         <is>
           <t>Entry price</t>
         </is>
       </c>
-      <c r="B5" s="28" t="n">
+      <c r="B5" s="29" t="n">
         <v>100</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="27" t="inlineStr">
+      <c r="A6" s="28" t="inlineStr">
         <is>
           <t>Stop loss</t>
         </is>
       </c>
-      <c r="B6" s="28" t="n">
+      <c r="B6" s="29" t="n">
         <v>92</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="27" t="inlineStr">
+      <c r="A7" s="28" t="inlineStr">
         <is>
           <t>Account / sleeve ₹</t>
         </is>
       </c>
-      <c r="B7" s="29" t="n">
+      <c r="B7" s="30" t="n">
         <v>263453</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="27" t="inlineStr">
+      <c r="A8" s="28" t="inlineStr">
         <is>
           <t>Risk budget %</t>
         </is>
       </c>
-      <c r="B8" s="30" t="n">
+      <c r="B8" s="31" t="n">
         <v>2</v>
       </c>
     </row>
@@ -5109,67 +5193,67 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="27" t="inlineStr">
+      <c r="A11" s="28" t="inlineStr">
         <is>
           <t>Risk per share</t>
         </is>
       </c>
-      <c r="B11" s="31">
+      <c r="B11" s="32">
         <f>B5-B6</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="27" t="inlineStr">
+      <c r="A12" s="28" t="inlineStr">
         <is>
           <t>Risk % of entry</t>
         </is>
       </c>
-      <c r="B12" s="32">
+      <c r="B12" s="33">
         <f>(B5-B6)/B5</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="27" t="inlineStr">
+      <c r="A13" s="28" t="inlineStr">
         <is>
           <t>Max ₹ at risk</t>
         </is>
       </c>
-      <c r="B13" s="33">
+      <c r="B13" s="34">
         <f>B7*B8/100</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="27" t="inlineStr">
+      <c r="A14" s="28" t="inlineStr">
         <is>
           <t>Max shares</t>
         </is>
       </c>
-      <c r="B14" s="33">
+      <c r="B14" s="34">
         <f>IF(B11&gt;0,FLOOR(B13/B11,1),0)</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="27" t="inlineStr">
+      <c r="A15" s="28" t="inlineStr">
         <is>
           <t>Capital required</t>
         </is>
       </c>
-      <c r="B15" s="33">
+      <c r="B15" s="34">
         <f>B14*B5</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="27" t="inlineStr">
+      <c r="A16" s="28" t="inlineStr">
         <is>
           <t>% of sleeve deployed</t>
         </is>
       </c>
-      <c r="B16" s="34">
+      <c r="B16" s="35">
         <f>IF(B7&gt;0,B15/B7,0)</f>
         <v/>
       </c>
@@ -5182,34 +5266,34 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="27" t="inlineStr">
+      <c r="A19" s="28" t="inlineStr">
         <is>
           <t>T1 pilot (25%)</t>
         </is>
       </c>
-      <c r="B19" s="33">
+      <c r="B19" s="34">
         <f>FLOOR(B14*0.25,1)</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="27" t="inlineStr">
+      <c r="A20" s="28" t="inlineStr">
         <is>
           <t>T2 core (50%)</t>
         </is>
       </c>
-      <c r="B20" s="33">
+      <c r="B20" s="34">
         <f>FLOOR(B14*0.5,1)</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="27" t="inlineStr">
+      <c r="A21" s="28" t="inlineStr">
         <is>
           <t>T3 final (25%)</t>
         </is>
       </c>
-      <c r="B21" s="33">
+      <c r="B21" s="34">
         <f>B14-B19-B20</f>
         <v/>
       </c>
@@ -5222,163 +5306,163 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="35" t="inlineStr">
+      <c r="A24" s="36" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="B24" s="35" t="inlineStr">
+      <c r="B24" s="36" t="inlineStr">
         <is>
           <t>Price</t>
         </is>
       </c>
-      <c r="C24" s="35" t="inlineStr">
+      <c r="C24" s="36" t="inlineStr">
         <is>
           <t>% of position</t>
         </is>
       </c>
-      <c r="D24" s="35" t="inlineStr">
+      <c r="D24" s="36" t="inlineStr">
         <is>
           <t>R:R</t>
         </is>
       </c>
-      <c r="E24" s="35" t="inlineStr">
+      <c r="E24" s="36" t="inlineStr">
         <is>
           <t>Reward %</t>
         </is>
       </c>
-      <c r="F24" s="35" t="inlineStr">
+      <c r="F24" s="36" t="inlineStr">
         <is>
           <t>P&amp;L ₹ (at max shares)</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="27" t="inlineStr">
+      <c r="A25" s="28" t="inlineStr">
         <is>
           <t>T1</t>
         </is>
       </c>
-      <c r="B25" s="28" t="n">
+      <c r="B25" s="29" t="n">
         <v>110</v>
       </c>
-      <c r="C25" s="36" t="n">
+      <c r="C25" s="37" t="n">
         <v>33</v>
       </c>
-      <c r="D25" s="37">
+      <c r="D25" s="38">
         <f>IF($B$5-$B$6&gt;0,(B25-$B$5)/($B$5-$B$6),0)</f>
         <v/>
       </c>
-      <c r="E25" s="34">
+      <c r="E25" s="35">
         <f>(B25-$B$5)/$B$5</f>
         <v/>
       </c>
-      <c r="F25" s="33">
+      <c r="F25" s="34">
         <f>(B25-$B$5)*FLOOR($B$14*C25/100,1)</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="27" t="inlineStr">
+      <c r="A26" s="28" t="inlineStr">
         <is>
           <t>T2</t>
         </is>
       </c>
-      <c r="B26" s="28" t="n">
+      <c r="B26" s="29" t="n">
         <v>120</v>
       </c>
-      <c r="C26" s="36" t="n">
+      <c r="C26" s="37" t="n">
         <v>33</v>
       </c>
-      <c r="D26" s="37">
+      <c r="D26" s="38">
         <f>IF($B$5-$B$6&gt;0,(B26-$B$5)/($B$5-$B$6),0)</f>
         <v/>
       </c>
-      <c r="E26" s="34">
+      <c r="E26" s="35">
         <f>(B26-$B$5)/$B$5</f>
         <v/>
       </c>
-      <c r="F26" s="33">
+      <c r="F26" s="34">
         <f>(B26-$B$5)*FLOOR($B$14*C26/100,1)</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="27" t="inlineStr">
+      <c r="A27" s="28" t="inlineStr">
         <is>
           <t>T3</t>
         </is>
       </c>
-      <c r="B27" s="28" t="n">
+      <c r="B27" s="29" t="n">
         <v>135</v>
       </c>
-      <c r="C27" s="36" t="n">
+      <c r="C27" s="37" t="n">
         <v>34</v>
       </c>
-      <c r="D27" s="37">
+      <c r="D27" s="38">
         <f>IF($B$5-$B$6&gt;0,(B27-$B$5)/($B$5-$B$6),0)</f>
         <v/>
       </c>
-      <c r="E27" s="34">
+      <c r="E27" s="35">
         <f>(B27-$B$5)/$B$5</f>
         <v/>
       </c>
-      <c r="F27" s="33">
+      <c r="F27" s="34">
         <f>(B27-$B$5)*FLOOR($B$14*C27/100,1)</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="38" t="inlineStr">
+      <c r="A28" s="39" t="inlineStr">
         <is>
           <t>Weighted avg R:R</t>
         </is>
       </c>
-      <c r="D28" s="37">
+      <c r="D28" s="38">
         <f>IF(SUM(C25:C27)&gt;0,SUMPRODUCT(D25:D27,C25:C27)/SUM(C25:C27),0)</f>
         <v/>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="38" t="inlineStr">
+      <c r="A29" s="39" t="inlineStr">
         <is>
           <t>Avg exit price</t>
         </is>
       </c>
-      <c r="B29" s="31">
+      <c r="B29" s="32">
         <f>IF(SUM(C25:C27)&gt;0,SUMPRODUCT(B25:B27,C25:C27)/SUM(C25:C27),0)</f>
         <v/>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="38" t="inlineStr">
+      <c r="A30" s="39" t="inlineStr">
         <is>
           <t>Full-run P&amp;L ₹</t>
         </is>
       </c>
-      <c r="B30" s="33">
+      <c r="B30" s="34">
         <f>SUM(F25:F27)</f>
         <v/>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="38" t="inlineStr">
+      <c r="A31" s="39" t="inlineStr">
         <is>
           <t>Payoff ratio (win/loss)</t>
         </is>
       </c>
-      <c r="B31" s="37">
+      <c r="B31" s="38">
         <f>IF(B13&gt;0,B30/B13,0)</f>
         <v/>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="38" t="inlineStr">
+      <c r="A32" s="39" t="inlineStr">
         <is>
           <t>Break-even win rate</t>
         </is>
       </c>
-      <c r="B32" s="34">
+      <c r="B32" s="35">
         <f>IF(B31&gt;0,1/(1+B31),0)</f>
         <v/>
       </c>
@@ -5506,7 +5590,7 @@
       <c r="I3" s="21" t="n">
         <v>30.59031517163864</v>
       </c>
-      <c r="J3" s="39" t="inlineStr">
+      <c r="J3" s="40" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -5551,7 +5635,7 @@
       <c r="I5" s="23" t="n">
         <v>-23.05421294278932</v>
       </c>
-      <c r="J5" s="40" t="inlineStr">
+      <c r="J5" s="41" t="inlineStr">
         <is>
           <t>HOLD_FOR_TLH</t>
         </is>
@@ -5588,7 +5672,7 @@
       <c r="G7" s="6" t="n"/>
       <c r="H7" s="6" t="n"/>
       <c r="I7" s="5" t="n"/>
-      <c r="J7" s="41" t="inlineStr">
+      <c r="J7" s="42" t="inlineStr">
         <is>
           <t>SOLD</t>
         </is>

</xml_diff>

<commit_message>
Confirm LPG fill: 7sh @ \$49.381, 2026-08-19
Buy order confirmed via INDmoney — order value \$345.67, avg price
\$49.381 (essentially identical to the \$49.39 reference used for sizing).
Risk \$9.67, right at the planned \$10 (1%) budget. Moved planned → open.

https://claude.ai/code/session_01HhF36NsLiVFyxhhXe4S24m
</commit_message>
<xml_diff>
--- a/examples/swing_monitor/Portfolio_Tracker.xlsx
+++ b/examples/swing_monitor/Portfolio_Tracker.xlsx
@@ -105,11 +105,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FEF3C7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00FEF9C3"/>
       </patternFill>
     </fill>
@@ -121,6 +116,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00DCFCE7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF3C7"/>
       </patternFill>
     </fill>
     <fill>
@@ -146,7 +146,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -174,23 +174,22 @@
     <xf numFmtId="3" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="169" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -576,7 +575,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-19 17:48  |  USD/INR 95.0  |  prices: override file (2026-08-12T10:29:00+00:00), yfinance off</t>
+          <t>Generated 2026-08-19 17:56  |  USD/INR 95.0  |  prices: override file (2026-08-12T10:29:00+00:00), yfinance off</t>
         </is>
       </c>
     </row>
@@ -3834,7 +3833,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:I28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3856,366 +3855,386 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>No open positions — flat.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>Entry</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>LTP</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>Next Target</t>
+        </is>
+      </c>
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>P&amp;L %</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>Risk ₹</t>
+        </is>
+      </c>
+      <c r="I2" s="4" t="inlineStr">
+        <is>
+          <t>Src</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>LPG</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="C3" s="5" t="n">
+        <v>49.381</v>
+      </c>
+      <c r="D3" s="5" t="n">
+        <v>49.39</v>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="F3" s="5" t="n">
+        <v>55</v>
+      </c>
+      <c r="G3" s="21" t="n">
+        <v>0.01822563334075156</v>
+      </c>
+      <c r="H3" s="5" t="n">
+        <v>9.667000000000002</v>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>override</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Planned Positions (staged, not filled)</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>No planned positions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Watchlist / Planned Entries</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>Plan Qty</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>Pilot Entry</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>LTP</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Trigger</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>Stop</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>Pivot</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>Dist to Buy Zone</t>
-        </is>
-      </c>
-      <c r="H5" s="4" t="inlineStr">
-        <is>
-          <t>Risk ₹ (full)</t>
-        </is>
-      </c>
-      <c r="I5" s="4" t="inlineStr">
-        <is>
-          <t>Src</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="25" t="inlineStr">
-        <is>
-          <t>LPG</t>
-        </is>
-      </c>
-      <c r="B6" s="25" t="n">
-        <v>7</v>
-      </c>
-      <c r="C6" s="25" t="n">
-        <v>49.39</v>
-      </c>
-      <c r="D6" s="25" t="n">
-        <v>49.39</v>
-      </c>
-      <c r="E6" s="25" t="n">
-        <v>48</v>
-      </c>
-      <c r="F6" s="25" t="n">
-        <v>48</v>
-      </c>
-      <c r="G6" s="25" t="inlineStr">
-        <is>
-          <t>IN ZONE</t>
-        </is>
-      </c>
-      <c r="H6" s="25" t="n">
-        <v>9.730000000000004</v>
-      </c>
-      <c r="I6" s="25" t="inlineStr">
-        <is>
-          <t>override</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>↳ LPG: Single clean entry ~7sh (not tranched, small account). Stop AT breakout pivot $48 per explicit choice — tight 2.8% stop, expect higher stop-out frequency than a wider stop in exchange for hard-capped $10 loss. Watch ceasefire news as a fundamental override signal independent of price action.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>Watchlist / Planned Entries</t>
-        </is>
-      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr"/>
+      <c r="F9" s="4" t="inlineStr"/>
+      <c r="G9" s="4" t="inlineStr"/>
+      <c r="H9" s="4" t="inlineStr"/>
+      <c r="I9" s="4" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Ticker</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>Trigger</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>Stop</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="inlineStr"/>
-      <c r="F10" s="4" t="inlineStr"/>
-      <c r="G10" s="4" t="inlineStr"/>
-      <c r="H10" s="4" t="inlineStr"/>
-      <c r="I10" s="4" t="inlineStr"/>
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>POLYCAB</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>₹9690 reclaim</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>₹9265</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>A- setup. Fresh box breakout to ATH 10,126, now pulling back. Enter 25% pilot on reclaim of 10D EMA 9,690. Add 50% above 10,126. Invalidate below 50D 9,265.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>POLYCAB</t>
+          <t>ACUTAAS</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>₹9690 reclaim</t>
+          <t>₹3333 pullback</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>₹9265</t>
+          <t>₹3070</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>A- setup. Fresh box breakout to ATH 10,126, now pulling back. Enter 25% pilot on reclaim of 10D EMA 9,690. Add 50% above 10,126. Invalidate below 50D 9,265.</t>
+          <t>WAIT — extended late-stage (box 5+), weekly reversal -4.9%. Only on orderly pullback to 21D ~3,333 holding. Never chase above 3,600.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>ACUTAAS</t>
+          <t>RSI</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>₹3333 pullback</t>
+          <t>$29.69-30.00</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>₹3070</t>
+          <t>$29.24</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>WAIT — extended late-stage (box 5+), weekly reversal -4.9%. Only on orderly pullback to 21D ~3,333 holding. Never chase above 3,600.</t>
+          <t>US gaming. Pullback entry to Darvas trail. Skip on close below 29.24.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>RSI</t>
+          <t>STX</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>$29.69-30.00</t>
+          <t>$475-510</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>$29.24</t>
+          <t>$448</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>US gaming. Pullback entry to Darvas trail. Skip on close below 29.24.</t>
+          <t>US semis. B+ setup — RE-CHECK after global chip selloff before acting.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>STX</t>
+          <t>WAAREEENER</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>$475-510</t>
+          <t>₹3080-3120</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>$448</t>
+          <t>₹2960</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>US semis. B+ setup — RE-CHECK after global chip selloff before acting.</t>
+          <t>B- setup. Wait for ATH &gt;3800.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>WAAREEENER</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>₹3080-3120</t>
+          <t>₹1280-1320</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>₹2960</t>
+          <t>₹1177</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>B- setup. Wait for ATH &gt;3800.</t>
+          <t>C+ setup — WAIT. Extended. Only on pullback to 10W EMA ~1280. Remove if closes below 21W 1177.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>₹1280-1320</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>₹1177</t>
-        </is>
-      </c>
+          <t>NIFTY</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr"/>
+      <c r="C16" s="5" t="inlineStr"/>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>C+ setup — WAIT. Extended. Only on pullback to 10W EMA ~1280. Remove if closes below 21W 1177.</t>
+          <t>RULE FIRED 2026-08-14: price 24,202 lost 21D EMA (24,326) AND 10D EMA (24,374) AND 150D SMA (24,294) AND 200D SMA (24,714) — only above 50D (24,124). Do not deploy new swing longs beyond pilot size until 21D EMA reclaimed.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>NIFTY</t>
+          <t>NIFTY500</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr"/>
       <c r="C17" s="5" t="inlineStr"/>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>RULE FIRED 2026-08-14: price 24,202 lost 21D EMA (24,326) AND 10D EMA (24,374) AND 150D SMA (24,294) AND 200D SMA (24,714) — only above 50D (24,124). Do not deploy new swing longs beyond pilot size until 21D EMA reclaimed.</t>
+          <t>Weaker but not broken: price 23,508 below 10D EMA (23,591) only, still above 21D/50D/150D/200D. Broader-market gauge for mid/small-cap names (more relevant than Nifty50 for names like NETWEB). RS vs Nasdaq at 11 (bottom decile), falling.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>NIFTY500</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr"/>
       <c r="C18" s="5" t="inlineStr"/>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Weaker but not broken: price 23,508 below 10D EMA (23,591) only, still above 21D/50D/150D/200D. Broader-market gauge for mid/small-cap names (more relevant than Nifty50 for names like NETWEB). RS vs Nasdaq at 11 (bottom decile), falling.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="inlineStr"/>
-      <c r="C19" s="5" t="inlineStr"/>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
           <t>US regime gauge — chip selloff in progress, watch for follow-through distribution</t>
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Closed Trade Journal</t>
+        </is>
+      </c>
+    </row>
     <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>Closed Trade Journal</t>
-        </is>
-      </c>
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Avg Entry</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>Avg Exit</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>P&amp;L %</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>Hold Days</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr"/>
+      <c r="I21" s="4" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="4" t="inlineStr">
-        <is>
-          <t>Ticker</t>
-        </is>
-      </c>
-      <c r="B22" s="4" t="inlineStr">
-        <is>
-          <t>Result</t>
-        </is>
-      </c>
-      <c r="C22" s="4" t="inlineStr">
-        <is>
-          <t>Avg Entry</t>
-        </is>
-      </c>
-      <c r="D22" s="4" t="inlineStr">
-        <is>
-          <t>Avg Exit</t>
-        </is>
-      </c>
-      <c r="E22" s="4" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
-      </c>
-      <c r="F22" s="4" t="inlineStr">
-        <is>
-          <t>P&amp;L %</t>
-        </is>
-      </c>
-      <c r="G22" s="4" t="inlineStr">
-        <is>
-          <t>Hold Days</t>
-        </is>
-      </c>
-      <c r="H22" s="4" t="inlineStr"/>
-      <c r="I22" s="4" t="inlineStr"/>
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>SNDK</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>profit</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="n">
+        <v>903.13</v>
+      </c>
+      <c r="D22" s="5" t="n">
+        <v>1250.83</v>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>$113</t>
+        </is>
+      </c>
+      <c r="F22" s="21" t="n">
+        <v>37.7</v>
+      </c>
+      <c r="G22" s="5" t="n">
+        <v>35</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>SNDK</t>
+          <t>BSE.NS</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
@@ -4224,85 +4243,85 @@
         </is>
       </c>
       <c r="C23" s="5" t="n">
-        <v>903.13</v>
+        <v>3415.5</v>
       </c>
       <c r="D23" s="5" t="n">
-        <v>1250.83</v>
+        <v>3994.53</v>
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>$113</t>
+          <t>₹4,632</t>
         </is>
       </c>
       <c r="F23" s="21" t="n">
-        <v>37.7</v>
+        <v>17</v>
       </c>
       <c r="G23" s="5" t="n">
-        <v>35</v>
+        <v>48</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>BSE.NS</t>
+          <t>KRN</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>profit</t>
+          <t>loss</t>
         </is>
       </c>
       <c r="C24" s="5" t="n">
-        <v>3415.5</v>
+        <v>1310</v>
       </c>
       <c r="D24" s="5" t="n">
-        <v>3994.53</v>
+        <v>1197.27</v>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>₹4,632</t>
-        </is>
-      </c>
-      <c r="F24" s="21" t="n">
-        <v>17</v>
+          <t>₹-2,480</t>
+        </is>
+      </c>
+      <c r="F24" s="23" t="n">
+        <v>-8.6</v>
       </c>
       <c r="G24" s="5" t="n">
-        <v>48</v>
+        <v>9</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>KRN</t>
+          <t>CPRX</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>loss</t>
+          <t>profit</t>
         </is>
       </c>
       <c r="C25" s="5" t="n">
-        <v>1310</v>
+        <v>28.03</v>
       </c>
       <c r="D25" s="5" t="n">
-        <v>1197.27</v>
+        <v>31.14</v>
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>₹-2,480</t>
-        </is>
-      </c>
-      <c r="F25" s="23" t="n">
-        <v>-8.6</v>
+          <t>$21</t>
+        </is>
+      </c>
+      <c r="F25" s="21" t="n">
+        <v>10.4</v>
       </c>
       <c r="G25" s="5" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>CPRX</t>
+          <t>ATHERENERG</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
@@ -4311,123 +4330,93 @@
         </is>
       </c>
       <c r="C26" s="5" t="n">
-        <v>28.03</v>
+        <v>960.4</v>
       </c>
       <c r="D26" s="5" t="n">
-        <v>31.14</v>
+        <v>979.5</v>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>$21</t>
+          <t>₹134</t>
         </is>
       </c>
       <c r="F26" s="21" t="n">
-        <v>10.4</v>
+        <v>2</v>
       </c>
       <c r="G26" s="5" t="n">
-        <v>14</v>
+        <v>37</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>ATHERENERG</t>
+          <t>LRCX</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>profit</t>
+          <t>scratch</t>
         </is>
       </c>
       <c r="C27" s="5" t="n">
-        <v>960.4</v>
+        <v>346.09</v>
       </c>
       <c r="D27" s="5" t="n">
-        <v>979.5</v>
+        <v>346</v>
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>₹134</t>
-        </is>
-      </c>
-      <c r="F27" s="21" t="n">
-        <v>2</v>
+          <t>$-0</t>
+        </is>
+      </c>
+      <c r="F27" s="23" t="n">
+        <v>-0.03</v>
       </c>
       <c r="G27" s="5" t="n">
-        <v>37</v>
+        <v>27</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>LRCX</t>
+          <t>DATAPATTNS</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>scratch</t>
+          <t>loss</t>
         </is>
       </c>
       <c r="C28" s="5" t="n">
-        <v>346.09</v>
+        <v>4805</v>
       </c>
       <c r="D28" s="5" t="n">
-        <v>346</v>
+        <v>4400</v>
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>$-0</t>
+          <t>₹-4,050</t>
         </is>
       </c>
       <c r="F28" s="23" t="n">
-        <v>-0.03</v>
-      </c>
-      <c r="G28" s="5" t="n">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="5" t="inlineStr">
-        <is>
-          <t>DATAPATTNS</t>
-        </is>
-      </c>
-      <c r="B29" s="5" t="inlineStr">
-        <is>
-          <t>loss</t>
-        </is>
-      </c>
-      <c r="C29" s="5" t="n">
-        <v>4805</v>
-      </c>
-      <c r="D29" s="5" t="n">
-        <v>4400</v>
-      </c>
-      <c r="E29" s="5" t="inlineStr">
-        <is>
-          <t>₹-4,050</t>
-        </is>
-      </c>
-      <c r="F29" s="23" t="n">
         <v>-8.4</v>
       </c>
-      <c r="G29" s="5" t="n"/>
+      <c r="G28" s="5" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="14">
-    <mergeCell ref="D19:I19"/>
-    <mergeCell ref="A7:I7"/>
+  <mergeCells count="13">
     <mergeCell ref="D11:I11"/>
+    <mergeCell ref="D10:I10"/>
     <mergeCell ref="D13:I13"/>
+    <mergeCell ref="A5:I5"/>
     <mergeCell ref="D14:I14"/>
     <mergeCell ref="D18:I18"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="D17:I17"/>
-    <mergeCell ref="A9:I9"/>
+    <mergeCell ref="A8:I8"/>
     <mergeCell ref="D12:I12"/>
     <mergeCell ref="D16:I16"/>
-    <mergeCell ref="A4:I4"/>
-    <mergeCell ref="A21:I21"/>
+    <mergeCell ref="A20:I20"/>
     <mergeCell ref="D15:I15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4566,7 +4555,7 @@
         <f>(H3-G3)*F3</f>
         <v/>
       </c>
-      <c r="K3" s="26">
+      <c r="K3" s="25">
         <f>IF(G3&gt;0,(H3-G3)/G3,0)</f>
         <v/>
       </c>
@@ -4615,7 +4604,7 @@
         <f>(H4-G4)*F4</f>
         <v/>
       </c>
-      <c r="K4" s="26">
+      <c r="K4" s="25">
         <f>IF(G4&gt;0,(H4-G4)/G4,0)</f>
         <v/>
       </c>
@@ -4664,7 +4653,7 @@
         <f>(H5-G5)*F5</f>
         <v/>
       </c>
-      <c r="K5" s="26">
+      <c r="K5" s="25">
         <f>IF(G5&gt;0,(H5-G5)/G5,0)</f>
         <v/>
       </c>
@@ -4713,7 +4702,7 @@
         <f>(H6-G6)*F6</f>
         <v/>
       </c>
-      <c r="K6" s="26">
+      <c r="K6" s="25">
         <f>IF(G6&gt;0,(H6-G6)/G6,0)</f>
         <v/>
       </c>
@@ -4762,7 +4751,7 @@
         <f>(H7-G7)*F7</f>
         <v/>
       </c>
-      <c r="K7" s="26">
+      <c r="K7" s="25">
         <f>IF(G7&gt;0,(H7-G7)/G7,0)</f>
         <v/>
       </c>
@@ -4811,7 +4800,7 @@
         <f>(H8-G8)*F8</f>
         <v/>
       </c>
-      <c r="K8" s="26">
+      <c r="K8" s="25">
         <f>IF(G8&gt;0,(H8-G8)/G8,0)</f>
         <v/>
       </c>
@@ -4860,7 +4849,7 @@
         <f>(H9-G9)*F9</f>
         <v/>
       </c>
-      <c r="K9" s="26">
+      <c r="K9" s="25">
         <f>IF(G9&gt;0,(H9-G9)/G9,0)</f>
         <v/>
       </c>
@@ -5125,7 +5114,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="27" t="inlineStr">
+      <c r="A1" s="26" t="inlineStr">
         <is>
           <t>POSITION SIZING &amp; R:R CALCULATOR</t>
         </is>
@@ -5146,42 +5135,42 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="28" t="inlineStr">
+      <c r="A5" s="27" t="inlineStr">
         <is>
           <t>Entry price</t>
         </is>
       </c>
-      <c r="B5" s="29" t="n">
+      <c r="B5" s="28" t="n">
         <v>100</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="28" t="inlineStr">
+      <c r="A6" s="27" t="inlineStr">
         <is>
           <t>Stop loss</t>
         </is>
       </c>
-      <c r="B6" s="29" t="n">
+      <c r="B6" s="28" t="n">
         <v>92</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="28" t="inlineStr">
+      <c r="A7" s="27" t="inlineStr">
         <is>
           <t>Account / sleeve ₹</t>
         </is>
       </c>
-      <c r="B7" s="30" t="n">
+      <c r="B7" s="29" t="n">
         <v>263453</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="28" t="inlineStr">
+      <c r="A8" s="27" t="inlineStr">
         <is>
           <t>Risk budget %</t>
         </is>
       </c>
-      <c r="B8" s="31" t="n">
+      <c r="B8" s="30" t="n">
         <v>2</v>
       </c>
     </row>
@@ -5193,67 +5182,67 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="28" t="inlineStr">
+      <c r="A11" s="27" t="inlineStr">
         <is>
           <t>Risk per share</t>
         </is>
       </c>
-      <c r="B11" s="32">
+      <c r="B11" s="31">
         <f>B5-B6</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="28" t="inlineStr">
+      <c r="A12" s="27" t="inlineStr">
         <is>
           <t>Risk % of entry</t>
         </is>
       </c>
-      <c r="B12" s="33">
+      <c r="B12" s="32">
         <f>(B5-B6)/B5</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="28" t="inlineStr">
+      <c r="A13" s="27" t="inlineStr">
         <is>
           <t>Max ₹ at risk</t>
         </is>
       </c>
-      <c r="B13" s="34">
+      <c r="B13" s="33">
         <f>B7*B8/100</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="28" t="inlineStr">
+      <c r="A14" s="27" t="inlineStr">
         <is>
           <t>Max shares</t>
         </is>
       </c>
-      <c r="B14" s="34">
+      <c r="B14" s="33">
         <f>IF(B11&gt;0,FLOOR(B13/B11,1),0)</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="28" t="inlineStr">
+      <c r="A15" s="27" t="inlineStr">
         <is>
           <t>Capital required</t>
         </is>
       </c>
-      <c r="B15" s="34">
+      <c r="B15" s="33">
         <f>B14*B5</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="28" t="inlineStr">
+      <c r="A16" s="27" t="inlineStr">
         <is>
           <t>% of sleeve deployed</t>
         </is>
       </c>
-      <c r="B16" s="35">
+      <c r="B16" s="34">
         <f>IF(B7&gt;0,B15/B7,0)</f>
         <v/>
       </c>
@@ -5266,34 +5255,34 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="28" t="inlineStr">
+      <c r="A19" s="27" t="inlineStr">
         <is>
           <t>T1 pilot (25%)</t>
         </is>
       </c>
-      <c r="B19" s="34">
+      <c r="B19" s="33">
         <f>FLOOR(B14*0.25,1)</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="28" t="inlineStr">
+      <c r="A20" s="27" t="inlineStr">
         <is>
           <t>T2 core (50%)</t>
         </is>
       </c>
-      <c r="B20" s="34">
+      <c r="B20" s="33">
         <f>FLOOR(B14*0.5,1)</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="28" t="inlineStr">
+      <c r="A21" s="27" t="inlineStr">
         <is>
           <t>T3 final (25%)</t>
         </is>
       </c>
-      <c r="B21" s="34">
+      <c r="B21" s="33">
         <f>B14-B19-B20</f>
         <v/>
       </c>
@@ -5306,163 +5295,163 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="36" t="inlineStr">
+      <c r="A24" s="35" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="B24" s="36" t="inlineStr">
+      <c r="B24" s="35" t="inlineStr">
         <is>
           <t>Price</t>
         </is>
       </c>
-      <c r="C24" s="36" t="inlineStr">
+      <c r="C24" s="35" t="inlineStr">
         <is>
           <t>% of position</t>
         </is>
       </c>
-      <c r="D24" s="36" t="inlineStr">
+      <c r="D24" s="35" t="inlineStr">
         <is>
           <t>R:R</t>
         </is>
       </c>
-      <c r="E24" s="36" t="inlineStr">
+      <c r="E24" s="35" t="inlineStr">
         <is>
           <t>Reward %</t>
         </is>
       </c>
-      <c r="F24" s="36" t="inlineStr">
+      <c r="F24" s="35" t="inlineStr">
         <is>
           <t>P&amp;L ₹ (at max shares)</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="28" t="inlineStr">
+      <c r="A25" s="27" t="inlineStr">
         <is>
           <t>T1</t>
         </is>
       </c>
-      <c r="B25" s="29" t="n">
+      <c r="B25" s="28" t="n">
         <v>110</v>
       </c>
-      <c r="C25" s="37" t="n">
+      <c r="C25" s="36" t="n">
         <v>33</v>
       </c>
-      <c r="D25" s="38">
+      <c r="D25" s="37">
         <f>IF($B$5-$B$6&gt;0,(B25-$B$5)/($B$5-$B$6),0)</f>
         <v/>
       </c>
-      <c r="E25" s="35">
+      <c r="E25" s="34">
         <f>(B25-$B$5)/$B$5</f>
         <v/>
       </c>
-      <c r="F25" s="34">
+      <c r="F25" s="33">
         <f>(B25-$B$5)*FLOOR($B$14*C25/100,1)</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="28" t="inlineStr">
+      <c r="A26" s="27" t="inlineStr">
         <is>
           <t>T2</t>
         </is>
       </c>
-      <c r="B26" s="29" t="n">
+      <c r="B26" s="28" t="n">
         <v>120</v>
       </c>
-      <c r="C26" s="37" t="n">
+      <c r="C26" s="36" t="n">
         <v>33</v>
       </c>
-      <c r="D26" s="38">
+      <c r="D26" s="37">
         <f>IF($B$5-$B$6&gt;0,(B26-$B$5)/($B$5-$B$6),0)</f>
         <v/>
       </c>
-      <c r="E26" s="35">
+      <c r="E26" s="34">
         <f>(B26-$B$5)/$B$5</f>
         <v/>
       </c>
-      <c r="F26" s="34">
+      <c r="F26" s="33">
         <f>(B26-$B$5)*FLOOR($B$14*C26/100,1)</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="28" t="inlineStr">
+      <c r="A27" s="27" t="inlineStr">
         <is>
           <t>T3</t>
         </is>
       </c>
-      <c r="B27" s="29" t="n">
+      <c r="B27" s="28" t="n">
         <v>135</v>
       </c>
-      <c r="C27" s="37" t="n">
+      <c r="C27" s="36" t="n">
         <v>34</v>
       </c>
-      <c r="D27" s="38">
+      <c r="D27" s="37">
         <f>IF($B$5-$B$6&gt;0,(B27-$B$5)/($B$5-$B$6),0)</f>
         <v/>
       </c>
-      <c r="E27" s="35">
+      <c r="E27" s="34">
         <f>(B27-$B$5)/$B$5</f>
         <v/>
       </c>
-      <c r="F27" s="34">
+      <c r="F27" s="33">
         <f>(B27-$B$5)*FLOOR($B$14*C27/100,1)</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="39" t="inlineStr">
+      <c r="A28" s="38" t="inlineStr">
         <is>
           <t>Weighted avg R:R</t>
         </is>
       </c>
-      <c r="D28" s="38">
+      <c r="D28" s="37">
         <f>IF(SUM(C25:C27)&gt;0,SUMPRODUCT(D25:D27,C25:C27)/SUM(C25:C27),0)</f>
         <v/>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="39" t="inlineStr">
+      <c r="A29" s="38" t="inlineStr">
         <is>
           <t>Avg exit price</t>
         </is>
       </c>
-      <c r="B29" s="32">
+      <c r="B29" s="31">
         <f>IF(SUM(C25:C27)&gt;0,SUMPRODUCT(B25:B27,C25:C27)/SUM(C25:C27),0)</f>
         <v/>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="39" t="inlineStr">
+      <c r="A30" s="38" t="inlineStr">
         <is>
           <t>Full-run P&amp;L ₹</t>
         </is>
       </c>
-      <c r="B30" s="34">
+      <c r="B30" s="33">
         <f>SUM(F25:F27)</f>
         <v/>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="39" t="inlineStr">
+      <c r="A31" s="38" t="inlineStr">
         <is>
           <t>Payoff ratio (win/loss)</t>
         </is>
       </c>
-      <c r="B31" s="38">
+      <c r="B31" s="37">
         <f>IF(B13&gt;0,B30/B13,0)</f>
         <v/>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="39" t="inlineStr">
+      <c r="A32" s="38" t="inlineStr">
         <is>
           <t>Break-even win rate</t>
         </is>
       </c>
-      <c r="B32" s="35">
+      <c r="B32" s="34">
         <f>IF(B31&gt;0,1/(1+B31),0)</f>
         <v/>
       </c>
@@ -5590,7 +5579,7 @@
       <c r="I3" s="21" t="n">
         <v>30.59031517163864</v>
       </c>
-      <c r="J3" s="40" t="inlineStr">
+      <c r="J3" s="39" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -5635,7 +5624,7 @@
       <c r="I5" s="23" t="n">
         <v>-23.05421294278932</v>
       </c>
-      <c r="J5" s="41" t="inlineStr">
+      <c r="J5" s="40" t="inlineStr">
         <is>
           <t>HOLD_FOR_TLH</t>
         </is>
@@ -5672,7 +5661,7 @@
       <c r="G7" s="6" t="n"/>
       <c r="H7" s="6" t="n"/>
       <c r="I7" s="5" t="n"/>
-      <c r="J7" s="42" t="inlineStr">
+      <c r="J7" s="41" t="inlineStr">
         <is>
           <t>SOLD</t>
         </is>

</xml_diff>

<commit_message>
Reverse NETWEB closure — stop never executed, position still open
Correction: NETWEB was logged as closed based on the assumption the SL-M
fired. It did not. The stock closed 5,065 the prior session — BELOW the
5,085 trigger — so an active stop would have executed. Strong evidence
the order was not live (likely DAY validity, expired, never re-placed).

Restored to swing_positions as open. Current 5,292.60 (+4.49%), position
near breakeven at -1.04% rather than the planned -4.92% loss. Added a
STOP_NOT_EXECUTED_ALERT block flagging that this is luck, not validation,
and that a hold/exit decision is required. Growth sleeve deployed figure
restored to 32,088.

https://claude.ai/code/session_01HhF36NsLiVFyxhhXe4S24m
</commit_message>
<xml_diff>
--- a/examples/swing_monitor/Portfolio_Tracker.xlsx
+++ b/examples/swing_monitor/Portfolio_Tracker.xlsx
@@ -575,7 +575,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-19 17:56  |  USD/INR 95.0  |  prices: override file (2026-08-12T10:29:00+00:00), yfinance off</t>
+          <t>Generated 2026-08-20 04:40  |  USD/INR 95.0  |  prices: override file (2026-08-12T10:29:00+00:00), yfinance off</t>
         </is>
       </c>
     </row>
@@ -5700,7 +5700,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Source: Colgate-Palmolive sale proceeds  |  Pool: ₹1,200,000  |  Risk/trade: 1%  |  Deployed: ₹0  |  Cash remaining: ₹1,198,422</t>
+          <t>Source: Colgate-Palmolive sale proceeds  |  Pool: ₹1,200,000  |  Risk/trade: 1%  |  Deployed: ₹32,088  |  Cash remaining: ₹1,167,912</t>
         </is>
       </c>
     </row>
@@ -5712,119 +5712,141 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>No active swing/growth positions.</t>
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Entry</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>LTP</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>Next Target</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>P&amp;L %</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>Risk ₹</t>
+        </is>
+      </c>
+      <c r="I15" s="4" t="inlineStr">
+        <is>
+          <t>Src</t>
+        </is>
+      </c>
+      <c r="J15" s="4" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>NETWEB</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="C16" s="13" t="n">
+        <v>5348</v>
+      </c>
+      <c r="D16" s="13" t="n">
+        <v>5292.6</v>
+      </c>
+      <c r="E16" s="13" t="n">
+        <v>5085</v>
+      </c>
+      <c r="F16" s="13" t="n">
+        <v>5800</v>
+      </c>
+      <c r="G16" s="23" t="n">
+        <v>-1.035901271503359</v>
+      </c>
+      <c r="H16" s="6" t="n">
+        <v>1578</v>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>override</t>
+        </is>
+      </c>
+      <c r="J16" s="5" t="inlineStr">
+        <is>
+          <t>open</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">↳ Notes: Original plan: reverse-pyramid 25-50-25, max risk 1% of growth_sleeve. Two clean options now: (A) honour the original stop and exit near breakeven (~-₹332), restarting on a fresh setup; or (B) consciously RE-UNDERWRITE as a new trade with a new stop and a restarted clock. Do NOT widen the stop below 5,085 — never widen a stop after entry. Core/Final tranches remain gated on Nifty 50 reclaiming its 21D EMA.
+</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>Planned Trades (redeployment of sale proceeds)</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>None yet — ~₹50L expected free after GILLETTE + COLPAL exits. Plan before redeploying.</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t>Closed Swing/Growth Journal</t>
         </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>Ticker</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>Result</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>Avg Entry</t>
-        </is>
-      </c>
-      <c r="D21" s="4" t="inlineStr">
-        <is>
-          <t>Avg Exit</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
-      </c>
-      <c r="F21" s="4" t="inlineStr">
-        <is>
-          <t>P&amp;L %</t>
-        </is>
-      </c>
-      <c r="G21" s="4" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="H21" s="4" t="inlineStr"/>
-      <c r="I21" s="4" t="inlineStr"/>
-      <c r="J21" s="4" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="5" t="inlineStr">
-        <is>
-          <t>NETWEB</t>
-        </is>
-      </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>loss</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="n">
-        <v>5348</v>
-      </c>
-      <c r="D22" s="5" t="n">
-        <v>5085</v>
-      </c>
-      <c r="E22" s="5" t="inlineStr">
-        <is>
-          <t>₹-1,578</t>
-        </is>
-      </c>
-      <c r="F22" s="23" t="n">
-        <v>-4.92</v>
-      </c>
-      <c r="G22" s="19" t="n">
-        <v>-1</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>↳ Stopped out via SL-M ~5,085 on a Nifty distribution day — stock down ~5% intraday from prior close on market-wide instability, not company-specific news. Exit price is an ESTIMATE (SL-M trigger level) — CONFIRM exact fill + exact date from the HDFC Securities contract note. Textbook outcome of the regime-gating call: the Nifty 50 21D EMA loss flagged the day before turned into exactly the kind of broad selloff that stops out pilot positions. Working stop (day-1-low based, tighter than the 4,825 structural level) did its job — loss capped at planned 0.13% of sleeve, no damage beyond the plan.</t>
+          <t>No closed swing/growth trades yet.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="9">
     <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A23:J23"/>
     <mergeCell ref="A14:J14"/>
+    <mergeCell ref="A22:J22"/>
     <mergeCell ref="A17:J17"/>
     <mergeCell ref="B8:J8"/>
-    <mergeCell ref="A20:J20"/>
     <mergeCell ref="B4:J4"/>
     <mergeCell ref="B6:J6"/>
+    <mergeCell ref="A19:J19"/>
     <mergeCell ref="A11:J11"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Confirm NETWEB GTD stop placed: trigger 5,085 / limit 5,050
Order confirmed placed (SL-M unsupported with GTD on this account, so
using SL with a 0.69% limit buffer — tighter than the ~1.5% ATR-based
buffer originally suggested; trades fill-price protection for slightly
higher non-fill risk on a violent gap). Logged the full history (first
attempt was DAY-validity and expired unnoticed, this is the corrected
GTD order) so the record explains why the position survived a stop
violation once already.

portfolio_tracker.py: Father tab's swing-position notes now also render
a history_note field, not just add_plan/notes.

https://claude.ai/code/session_01HhF36NsLiVFyxhhXe4S24m
</commit_message>
<xml_diff>
--- a/examples/swing_monitor/Portfolio_Tracker.xlsx
+++ b/examples/swing_monitor/Portfolio_Tracker.xlsx
@@ -575,7 +575,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-20 04:40  |  USD/INR 95.0  |  prices: override file (2026-08-12T10:29:00+00:00), yfinance off</t>
+          <t>Generated 2026-08-20 04:57  |  USD/INR 95.0  |  prices: override file (2026-08-12T10:29:00+00:00), yfinance off</t>
         </is>
       </c>
     </row>
@@ -5473,7 +5473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J23"/>
+  <dimension ref="A1:J24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5804,49 +5804,57 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">↳ Notes: Original plan: reverse-pyramid 25-50-25, max risk 1% of growth_sleeve. Two clean options now: (A) honour the original stop and exit near breakeven (~-₹332), restarting on a fresh setup; or (B) consciously RE-UNDERWRITE as a new trade with a new stop and a restarted clock. Do NOT widen the stop below 5,085 — never widen a stop after entry. Core/Final tranches remain gated on Nifty 50 reclaiming its 21D EMA.
+          <t xml:space="preserve">↳ History: 2026-08-20: First SL-M attempt never fired (was DAY-validity, expired unnoticed) — stock traded through 5,085 on a closing basis and the position stayed open by accident, not by design. Re-underwritten in place: same 5,085 stop level, now a proper GTD SL order (trigger 5,085 / limit 5,050, ~0.69% buffer — tighter than the ~1.5% ATR-based buffer originally suggested; protects fill price, slightly raises non-fill risk on a violent gap — check the order book at open on any sharp down-day). CONFIRM this order shows ACTIVE in HDFC Securities' order book, not just "placed."
 </t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>↳ Notes: Reverse-pyramid / 25-50-25 plan. Do NOT widen the stop below 5,085. Core/Final tranches remain gated on Nifty 50 reclaiming its 21D EMA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
         <is>
           <t>Planned Trades (redeployment of sale proceeds)</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>None yet — ~₹50L expected free after GILLETTE + COLPAL exits. Plan before redeploying.</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>Closed Swing/Growth Journal</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>No closed swing/growth trades yet.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="10">
     <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A23:J23"/>
     <mergeCell ref="A14:J14"/>
-    <mergeCell ref="A22:J22"/>
     <mergeCell ref="A17:J17"/>
+    <mergeCell ref="A18:J18"/>
     <mergeCell ref="B8:J8"/>
+    <mergeCell ref="A20:J20"/>
     <mergeCell ref="B4:J4"/>
     <mergeCell ref="B6:J6"/>
-    <mergeCell ref="A19:J19"/>
     <mergeCell ref="A11:J11"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Log DATAPATTNS buy-stop order: trigger 4,830 / limit 4,895 / 11sh
Pilot-sized entry order placed (GTD through tomorrow), pending fill.
Flagged as a smaller/earlier confirmation than the original plan's
Core-tranche gate (close above 4,955.90 ATH) — this targets an R1 pivot
reclaim after yesterday's pullback, not a confirmed breakout. Volume
badge clarified as weekly not single-day, weaker signal than first read.

Protective stop (4,700 trigger / 4,650 limit) NOT yet placed — explicitly
flagged to queue the instant a fill confirms, given the NETWEB history of
an unprotected position surviving a stop violation by accident.

Confirmed NETWEB's GTD stop now shows active in the HDFC order book.

https://claude.ai/code/session_01HhF36NsLiVFyxhhXe4S24m
</commit_message>
<xml_diff>
--- a/examples/swing_monitor/Portfolio_Tracker.xlsx
+++ b/examples/swing_monitor/Portfolio_Tracker.xlsx
@@ -575,7 +575,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-20 04:57  |  USD/INR 95.0  |  prices: override file (2026-08-12T10:29:00+00:00), yfinance off</t>
+          <t>Generated 2026-08-20 05:05  |  USD/INR 95.0  |  prices: override file (2026-08-12T10:29:00+00:00), yfinance off</t>
         </is>
       </c>
     </row>
@@ -5473,7 +5473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J24"/>
+  <dimension ref="A1:J27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5816,44 +5816,99 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>DATAPATTNS</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="C19" s="13" t="n">
+        <v>4830</v>
+      </c>
+      <c r="D19" s="13" t="n">
+        <v>4787</v>
+      </c>
+      <c r="E19" s="13" t="n">
+        <v>4700</v>
+      </c>
+      <c r="F19" s="13" t="n">
+        <v>4955.9</v>
+      </c>
+      <c r="G19" s="23" t="n">
+        <v>-0.8902691511387117</v>
+      </c>
+      <c r="H19" s="6" t="n">
+        <v>1430</v>
+      </c>
+      <c r="I19" s="5" t="inlineStr">
+        <is>
+          <t>override</t>
+        </is>
+      </c>
+      <c r="J19" s="5" t="inlineStr">
+        <is>
+          <t>order_pending</t>
+        </is>
+      </c>
+    </row>
     <row r="20">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>Planned Trades (redeployment of sale proceeds)</t>
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">↳ History: 2026-08-19/20: Spiked to 'Buy Zone' tag, vol badge later clarified as a WEEKLY (not single-day) comparison — weaker confirmation than first read. Gave back most of the spike next session (pulled back to ~4785-4790). This buy-stop (4830) targets a smaller R1-pivot reclaim, not a reclaim of the prior high (4918) or the original Core-tranche gate (4955.90 ATH). Pilot-sized (11sh matches the original 25% tranche), so risk is small even if this doesn't pan out — but treat this as a speculative "buying the first reclaim after a pullback" entry, not a confirmed-breakout buy.
+</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>None yet — ~₹50L expected free after GILLETTE + COLPAL exits. Plan before redeploying.</t>
+          <t>↳ Notes: STOP NOT YET LIVE. The instant a fill confirms, place GTD SL trigger 4,700 / limit 4,650 same session — do not leave overnight unprotected (see NETWEB history for why this matters).</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>Closed Swing/Growth Journal</t>
+          <t>Planned Trades (redeployment of sale proceeds)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
+          <t>None yet — ~₹50L expected free after GILLETTE + COLPAL exits. Plan before redeploying.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>Closed Swing/Growth Journal</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
           <t>No closed swing/growth trades yet.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="12">
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A23:J23"/>
     <mergeCell ref="A14:J14"/>
     <mergeCell ref="A17:J17"/>
     <mergeCell ref="A18:J18"/>
+    <mergeCell ref="A21:J21"/>
     <mergeCell ref="B8:J8"/>
     <mergeCell ref="A20:J20"/>
     <mergeCell ref="B4:J4"/>
+    <mergeCell ref="A26:J26"/>
     <mergeCell ref="B6:J6"/>
     <mergeCell ref="A11:J11"/>
   </mergeCells>

</xml_diff>

<commit_message>
Revise DATAPATTNS order: trigger raised 4,830 -> 4,895, limit -> 4,950
Better confirmation level — reclaims the actual Buy Zone session price
(4,894.85), not just a minor R1 pivot. Still below the 4,955.90 ATH/Core
gate, still pilot-sized (11sh). Stop level held at 4,700 unchanged
(technical support, not adjusted for the higher entry). GTD extended
through 2026-08-22.

https://claude.ai/code/session_01HhF36NsLiVFyxhhXe4S24m
</commit_message>
<xml_diff>
--- a/examples/swing_monitor/Portfolio_Tracker.xlsx
+++ b/examples/swing_monitor/Portfolio_Tracker.xlsx
@@ -575,7 +575,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-20 05:05  |  USD/INR 95.0  |  prices: override file (2026-08-12T10:29:00+00:00), yfinance off</t>
+          <t>Generated 2026-08-20 05:10  |  USD/INR 95.0  |  prices: override file (2026-08-12T10:29:00+00:00), yfinance off</t>
         </is>
       </c>
     </row>
@@ -5826,7 +5826,7 @@
         <v>11</v>
       </c>
       <c r="C19" s="13" t="n">
-        <v>4830</v>
+        <v>4895</v>
       </c>
       <c r="D19" s="13" t="n">
         <v>4787</v>
@@ -5838,10 +5838,10 @@
         <v>4955.9</v>
       </c>
       <c r="G19" s="23" t="n">
-        <v>-0.8902691511387117</v>
+        <v>-2.206332992849847</v>
       </c>
       <c r="H19" s="6" t="n">
-        <v>1430</v>
+        <v>2145</v>
       </c>
       <c r="I19" s="5" t="inlineStr">
         <is>
@@ -5857,7 +5857,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">↳ History: 2026-08-19/20: Spiked to 'Buy Zone' tag, vol badge later clarified as a WEEKLY (not single-day) comparison — weaker confirmation than first read. Gave back most of the spike next session (pulled back to ~4785-4790). This buy-stop (4830) targets a smaller R1-pivot reclaim, not a reclaim of the prior high (4918) or the original Core-tranche gate (4955.90 ATH). Pilot-sized (11sh matches the original 25% tranche), so risk is small even if this doesn't pan out — but treat this as a speculative "buying the first reclaim after a pullback" entry, not a confirmed-breakout buy.
+          <t xml:space="preserve">↳ History: 2026-08-19/20: Spiked to 'Buy Zone' tag at 4,894.85, vol badge later clarified as a WEEKLY (not single-day) comparison — weaker confirmation than first read. Gave back most of the spike next session (pulled back to ~4785-4790). 2026-08-20: First order (trigger 4,830, R1 pivot reclaim) revised UP to trigger 4,895 / limit 4,950 — now requires reclaiming the actual Buy Zone session price, not just a minor pivot. Better confirmation, still below the 4,955.90 ATH/Core gate. Pilot-sized (11sh, matches the original 25% tranche) — risk to the 4,700 stop is 0.18-0.23% of sleeve regardless of exact fill price. Stop level unchanged at 4,700 (technical support, not adjusted for entry price).
 </t>
         </is>
       </c>

</xml_diff>

<commit_message>
Confirm DATAPATTNS filled at 4,895, stop placed same session
Entry filled at trigger (4,895 x 11sh, no slippage into the limit).
Protective GTD SL placed immediately (trigger 4,700 / limit 4,650) —
correct discipline, entry and protection in the same sitting, unlike
the NETWEB gap. Growth sleeve now shows both positions live: deployed
85,933 / cash 1,114,067.

https://claude.ai/code/session_01HhF36NsLiVFyxhhXe4S24m
</commit_message>
<xml_diff>
--- a/examples/swing_monitor/Portfolio_Tracker.xlsx
+++ b/examples/swing_monitor/Portfolio_Tracker.xlsx
@@ -575,7 +575,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-20 05:10  |  USD/INR 95.0  |  prices: override file (2026-08-12T10:29:00+00:00), yfinance off</t>
+          <t>Generated 2026-08-21 05:37  |  USD/INR 95.0  |  prices: override file (2026-08-12T10:29:00+00:00), yfinance off</t>
         </is>
       </c>
     </row>
@@ -5700,7 +5700,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Source: Colgate-Palmolive sale proceeds  |  Pool: ₹1,200,000  |  Risk/trade: 1%  |  Deployed: ₹32,088  |  Cash remaining: ₹1,167,912</t>
+          <t>Source: Colgate-Palmolive sale proceeds  |  Pool: ₹1,200,000  |  Risk/trade: 1%  |  Deployed: ₹85,933  |  Cash remaining: ₹1,114,067</t>
         </is>
       </c>
     </row>
@@ -5829,7 +5829,7 @@
         <v>4895</v>
       </c>
       <c r="D19" s="13" t="n">
-        <v>4787</v>
+        <v>4895</v>
       </c>
       <c r="E19" s="13" t="n">
         <v>4700</v>
@@ -5837,8 +5837,8 @@
       <c r="F19" s="13" t="n">
         <v>4955.9</v>
       </c>
-      <c r="G19" s="23" t="n">
-        <v>-2.206332992849847</v>
+      <c r="G19" s="21" t="n">
+        <v>0</v>
       </c>
       <c r="H19" s="6" t="n">
         <v>2145</v>
@@ -5850,7 +5850,7 @@
       </c>
       <c r="J19" s="5" t="inlineStr">
         <is>
-          <t>order_pending</t>
+          <t>open</t>
         </is>
       </c>
     </row>
@@ -5865,7 +5865,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>↳ Notes: STOP NOT YET LIVE. The instant a fill confirms, place GTD SL trigger 4,700 / limit 4,650 same session — do not leave overnight unprotected (see NETWEB history for why this matters).</t>
+          <t>↳ Notes: Reverse-pyramid / 25-50-25 plan. Pilot filled + protected same session — correct discipline, matches the NETWEB lesson. Core (23sh) still gated on close above 4,955.90 ATH on volume + Nifty 50 21D EMA reclaim.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Close LPG (Vishesh) and DATAPATTNS (father) — both stopped out
LPG: same-day whipsaw, entry and stop both 2026-08-19. Exit $48.21
(slightly better than the $48.00 trigger). Loss $8.20 (-2.37%), close
to the tight 2.8%-stop plan. Clean execution, confirmed via order
history screenshot.

DATAPATTNS: exit at the GTD SL limit price ₹4,650, confirmed by user
verbally — exact date pending contract note (placeholder). Loss ₹2,695
(-5.01%), landed right at the planned stop distance. Second consecutive
loss on this stock (first was June, -8.4%) — flagged in the post-mortem
as a pattern worth extra skepticism on any future setup regardless of
chart quality.

Growth sleeve now shows only NETWEB deployed (₹32,088); cash updated to
reflect DATAPATTNS's realized loss. Vishesh's own swing book is flat.

https://claude.ai/code/session_01HhF36NsLiVFyxhhXe4S24m
</commit_message>
<xml_diff>
--- a/examples/swing_monitor/Portfolio_Tracker.xlsx
+++ b/examples/swing_monitor/Portfolio_Tracker.xlsx
@@ -575,7 +575,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-21 05:37  |  USD/INR 95.0  |  prices: override file (2026-08-12T10:29:00+00:00), yfinance off</t>
+          <t>Generated 2026-08-26 16:42  |  USD/INR 95.0  |  prices: override file (2026-08-12T10:29:00+00:00), yfinance off</t>
         </is>
       </c>
     </row>
@@ -3833,7 +3833,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I28"/>
+  <dimension ref="A1:I42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3855,569 +3855,719 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>No open positions — flat.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Planned Positions (staged, not filled)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>No planned positions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Watchlist / Planned Entries</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>Qty</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>Entry</t>
-        </is>
-      </c>
-      <c r="D2" s="4" t="inlineStr">
-        <is>
-          <t>LTP</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Trigger</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>Stop</t>
         </is>
       </c>
-      <c r="F2" s="4" t="inlineStr">
-        <is>
-          <t>Next Target</t>
-        </is>
-      </c>
-      <c r="G2" s="4" t="inlineStr">
-        <is>
-          <t>P&amp;L %</t>
-        </is>
-      </c>
-      <c r="H2" s="4" t="inlineStr">
-        <is>
-          <t>Risk ₹</t>
-        </is>
-      </c>
-      <c r="I2" s="4" t="inlineStr">
-        <is>
-          <t>Src</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>LPG</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="n">
-        <v>7</v>
-      </c>
-      <c r="C3" s="5" t="n">
-        <v>49.381</v>
-      </c>
-      <c r="D3" s="5" t="n">
-        <v>49.39</v>
-      </c>
-      <c r="E3" s="5" t="n">
-        <v>48</v>
-      </c>
-      <c r="F3" s="5" t="n">
-        <v>55</v>
-      </c>
-      <c r="G3" s="21" t="n">
-        <v>0.01822563334075156</v>
-      </c>
-      <c r="H3" s="5" t="n">
-        <v>9.667000000000002</v>
-      </c>
-      <c r="I3" s="5" t="inlineStr">
-        <is>
-          <t>override</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>Planned Positions (staged, not filled)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>No planned positions.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>Watchlist / Planned Entries</t>
-        </is>
-      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr"/>
+      <c r="F8" s="4" t="inlineStr"/>
+      <c r="G8" s="4" t="inlineStr"/>
+      <c r="H8" s="4" t="inlineStr"/>
+      <c r="I8" s="4" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>Ticker</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>Trigger</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>Stop</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="inlineStr"/>
-      <c r="F9" s="4" t="inlineStr"/>
-      <c r="G9" s="4" t="inlineStr"/>
-      <c r="H9" s="4" t="inlineStr"/>
-      <c r="I9" s="4" t="inlineStr"/>
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>ACUTAAS</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>₹3333 pullback</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>₹3070</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>WAIT — extended late-stage (box 5+), weekly reversal -4.9%. Only on orderly pullback to 21D ~3,333 holding. Never chase above 3,600.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>POLYCAB</t>
+          <t>RSI</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>₹9690 reclaim</t>
+          <t>$29.69-30.00</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>₹9265</t>
+          <t>$29.24</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>A- setup. Fresh box breakout to ATH 10,126, now pulling back. Enter 25% pilot on reclaim of 10D EMA 9,690. Add 50% above 10,126. Invalidate below 50D 9,265.</t>
+          <t>US gaming. Pullback entry to Darvas trail. Skip on close below 29.24.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>ACUTAAS</t>
+          <t>STX</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>₹3333 pullback</t>
+          <t>$475-510</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>₹3070</t>
+          <t>$448</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>WAIT — extended late-stage (box 5+), weekly reversal -4.9%. Only on orderly pullback to 21D ~3,333 holding. Never chase above 3,600.</t>
+          <t>US semis. B+ setup — RE-CHECK after global chip selloff before acting.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>RSI</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>$29.69-30.00</t>
+          <t>₹1280-1320</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>$29.24</t>
+          <t>₹1177</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>US gaming. Pullback entry to Darvas trail. Skip on close below 29.24.</t>
+          <t>C+ setup — WAIT. Extended. Only on pullback to 10W EMA ~1280. Remove if closes below 21W 1177.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>STX</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>$475-510</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>$448</t>
-        </is>
-      </c>
+          <t>NIFTY</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr"/>
+      <c r="C13" s="5" t="inlineStr"/>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>US semis. B+ setup — RE-CHECK after global chip selloff before acting.</t>
+          <t>RULE FIRED 2026-08-14: price 24,202 lost 21D EMA (24,326) AND 10D EMA (24,374) AND 150D SMA (24,294) AND 200D SMA (24,714) — only above 50D (24,124). Do not deploy new swing longs beyond pilot size until 21D EMA reclaimed.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>WAAREEENER</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>₹3080-3120</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>₹2960</t>
-        </is>
-      </c>
+          <t>NIFTY500</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr"/>
+      <c r="C14" s="5" t="inlineStr"/>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>B- setup. Wait for ATH &gt;3800.</t>
+          <t>Weaker but not broken: price 23,508 below 10D EMA (23,591) only, still above 21D/50D/150D/200D. Broader-market gauge for mid/small-cap names (more relevant than Nifty50 for names like NETWEB). RS vs Nasdaq at 11 (bottom decile), falling.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>₹1280-1320</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>₹1177</t>
-        </is>
-      </c>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr"/>
+      <c r="C15" s="5" t="inlineStr"/>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>C+ setup — WAIT. Extended. Only on pullback to 10W EMA ~1280. Remove if closes below 21W 1177.</t>
+          <t>US regime gauge — chip selloff in progress, watch for follow-through distribution</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>NIFTY</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr"/>
       <c r="C16" s="5" t="inlineStr"/>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>RULE FIRED 2026-08-14: price 24,202 lost 21D EMA (24,326) AND 10D EMA (24,374) AND 150D SMA (24,294) AND 200D SMA (24,714) — only above 50D (24,124). Do not deploy new swing longs beyond pilot size until 21D EMA reclaimed.</t>
+          <t>From TradingView 'Breaking Out' follow list, 2026-08-24. No analysis yet — pending review.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>NIFTY500</t>
+          <t>ATUSF</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr"/>
       <c r="C17" s="5" t="inlineStr"/>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Weaker but not broken: price 23,508 below 10D EMA (23,591) only, still above 21D/50D/150D/200D. Broader-market gauge for mid/small-cap names (more relevant than Nifty50 for names like NETWEB). RS vs Nasdaq at 11 (bottom decile), falling.</t>
+          <t>From TradingView 'Breaking Out' follow list, 2026-08-24. Ticker/company identity unconfirmed (OTC-style suffix) — verify before analysis. No analysis yet.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>LRCX</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr"/>
       <c r="C18" s="5" t="inlineStr"/>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>US regime gauge — chip selloff in progress, watch for follow-through distribution</t>
+          <t>From TradingView follow list, 2026-08-24. Previously closed swing (entry 346, scratch exit). Re-following, not re-entered. No fresh analysis yet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>SNDK</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr"/>
+      <c r="C19" s="5" t="inlineStr"/>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>From TradingView follow list, 2026-08-24. Previously closed swing (+37.7%). Re-following. No fresh analysis yet.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>Closed Trade Journal</t>
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr"/>
+      <c r="C20" s="5" t="inlineStr"/>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>From TradingView follow list, 2026-08-24. No analysis yet — pending review.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>Ticker</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>Result</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>Avg Entry</t>
-        </is>
-      </c>
-      <c r="D21" s="4" t="inlineStr">
-        <is>
-          <t>Avg Exit</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
-      </c>
-      <c r="F21" s="4" t="inlineStr">
-        <is>
-          <t>P&amp;L %</t>
-        </is>
-      </c>
-      <c r="G21" s="4" t="inlineStr">
-        <is>
-          <t>Hold Days</t>
-        </is>
-      </c>
-      <c r="H21" s="4" t="inlineStr"/>
-      <c r="I21" s="4" t="inlineStr"/>
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>INTC</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr"/>
+      <c r="C21" s="5" t="inlineStr"/>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>From TradingView follow list, 2026-08-24. No analysis yet — pending review.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>SNDK</t>
-        </is>
-      </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>profit</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="n">
-        <v>903.13</v>
-      </c>
-      <c r="D22" s="5" t="n">
-        <v>1250.83</v>
-      </c>
-      <c r="E22" s="5" t="inlineStr">
-        <is>
-          <t>$113</t>
-        </is>
-      </c>
-      <c r="F22" s="21" t="n">
-        <v>37.7</v>
-      </c>
-      <c r="G22" s="5" t="n">
-        <v>35</v>
+          <t>OUST</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr"/>
+      <c r="C22" s="5" t="inlineStr"/>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>From TradingView follow list, 2026-08-24. No analysis yet — pending review.</t>
+        </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>BSE.NS</t>
-        </is>
-      </c>
-      <c r="B23" s="5" t="inlineStr">
-        <is>
-          <t>profit</t>
-        </is>
-      </c>
-      <c r="C23" s="5" t="n">
-        <v>3415.5</v>
-      </c>
-      <c r="D23" s="5" t="n">
-        <v>3994.53</v>
-      </c>
-      <c r="E23" s="5" t="inlineStr">
-        <is>
-          <t>₹4,632</t>
-        </is>
-      </c>
-      <c r="F23" s="21" t="n">
-        <v>17</v>
-      </c>
-      <c r="G23" s="5" t="n">
-        <v>48</v>
+          <t>CGNX</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr"/>
+      <c r="C23" s="5" t="inlineStr"/>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>From TradingView follow list, 2026-08-24. No analysis yet — pending review.</t>
+        </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>KRN</t>
-        </is>
-      </c>
-      <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t>loss</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="n">
-        <v>1310</v>
-      </c>
-      <c r="D24" s="5" t="n">
-        <v>1197.27</v>
-      </c>
-      <c r="E24" s="5" t="inlineStr">
-        <is>
-          <t>₹-2,480</t>
-        </is>
-      </c>
-      <c r="F24" s="23" t="n">
-        <v>-8.6</v>
-      </c>
-      <c r="G24" s="5" t="n">
-        <v>9</v>
+          <t>KALYANKJIL</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr"/>
+      <c r="C24" s="5" t="inlineStr"/>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Kalyan Jewellers India. From TradingView follow list, 2026-08-24. No analysis yet — pending review.</t>
+        </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>CPRX</t>
-        </is>
-      </c>
-      <c r="B25" s="5" t="inlineStr">
-        <is>
-          <t>profit</t>
-        </is>
-      </c>
-      <c r="C25" s="5" t="n">
-        <v>28.03</v>
-      </c>
-      <c r="D25" s="5" t="n">
-        <v>31.14</v>
-      </c>
-      <c r="E25" s="5" t="inlineStr">
-        <is>
-          <t>$21</t>
-        </is>
-      </c>
-      <c r="F25" s="21" t="n">
-        <v>10.4</v>
-      </c>
-      <c r="G25" s="5" t="n">
-        <v>14</v>
+          <t>RAINBOW</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr"/>
+      <c r="C25" s="5" t="inlineStr"/>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Rainbow Childrens Medicare. From TradingView follow list, 2026-08-24. No analysis yet — pending review.</t>
+        </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>ATHERENERG</t>
-        </is>
-      </c>
-      <c r="B26" s="5" t="inlineStr">
-        <is>
-          <t>profit</t>
-        </is>
-      </c>
-      <c r="C26" s="5" t="n">
-        <v>960.4</v>
-      </c>
-      <c r="D26" s="5" t="n">
-        <v>979.5</v>
-      </c>
-      <c r="E26" s="5" t="inlineStr">
-        <is>
-          <t>₹134</t>
-        </is>
-      </c>
-      <c r="F26" s="21" t="n">
-        <v>2</v>
-      </c>
-      <c r="G26" s="5" t="n">
-        <v>37</v>
+          <t>AUROPHARMA</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr"/>
+      <c r="C26" s="5" t="inlineStr"/>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Aurobindo Pharma. From TradingView follow list, 2026-08-24. No analysis yet — pending review.</t>
+        </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>LRCX</t>
-        </is>
-      </c>
-      <c r="B27" s="5" t="inlineStr">
-        <is>
-          <t>scratch</t>
-        </is>
-      </c>
-      <c r="C27" s="5" t="n">
-        <v>346.09</v>
-      </c>
-      <c r="D27" s="5" t="n">
-        <v>346</v>
-      </c>
-      <c r="E27" s="5" t="inlineStr">
-        <is>
-          <t>$-0</t>
-        </is>
-      </c>
-      <c r="F27" s="23" t="n">
-        <v>-0.03</v>
-      </c>
-      <c r="G27" s="5" t="n">
-        <v>27</v>
+          <t>ATHERENERG</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr"/>
+      <c r="C27" s="5" t="inlineStr"/>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Ather Energy. From TradingView follow list, 2026-08-24. Previously closed swing (+2.0%). Re-following, not re-entered. No fresh analysis yet.</t>
+        </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
+          <t>NEULANDLAB</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr"/>
+      <c r="C28" s="5" t="inlineStr"/>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Neuland Laboratories. From TradingView follow list, 2026-08-24. No analysis yet — pending review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>SANDHAR</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr"/>
+      <c r="C29" s="5" t="inlineStr"/>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Sandhar Technologies. From TradingView follow list, 2026-08-24. No analysis yet — pending review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>CGPOWER</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr"/>
+      <c r="C30" s="5" t="inlineStr"/>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>CG Power &amp; Industrial Solutions. From TradingView follow list, 2026-08-24. No analysis yet — pending review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>KERNEX</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr"/>
+      <c r="C31" s="5" t="inlineStr"/>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Name partially visible in screenshot (cut off) — likely Kernex Microsystems, CONFIRM. From TradingView follow list, 2026-08-24. No analysis yet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>Closed Trade Journal</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>Avg Entry</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>Avg Exit</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t>P&amp;L %</t>
+        </is>
+      </c>
+      <c r="G34" s="4" t="inlineStr">
+        <is>
+          <t>Hold Days</t>
+        </is>
+      </c>
+      <c r="H34" s="4" t="inlineStr"/>
+      <c r="I34" s="4" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>LPG</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>loss</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="n">
+        <v>49.381</v>
+      </c>
+      <c r="D35" s="5" t="n">
+        <v>48.21</v>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>$-8</t>
+        </is>
+      </c>
+      <c r="F35" s="23" t="n">
+        <v>-2.37</v>
+      </c>
+      <c r="G35" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>SNDK</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>profit</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="n">
+        <v>903.13</v>
+      </c>
+      <c r="D36" s="5" t="n">
+        <v>1250.83</v>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>$113</t>
+        </is>
+      </c>
+      <c r="F36" s="21" t="n">
+        <v>37.7</v>
+      </c>
+      <c r="G36" s="5" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>BSE.NS</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>profit</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="n">
+        <v>3415.5</v>
+      </c>
+      <c r="D37" s="5" t="n">
+        <v>3994.53</v>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>₹4,632</t>
+        </is>
+      </c>
+      <c r="F37" s="21" t="n">
+        <v>17</v>
+      </c>
+      <c r="G37" s="5" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>KRN</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>loss</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="n">
+        <v>1310</v>
+      </c>
+      <c r="D38" s="5" t="n">
+        <v>1197.27</v>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>₹-2,480</t>
+        </is>
+      </c>
+      <c r="F38" s="23" t="n">
+        <v>-8.6</v>
+      </c>
+      <c r="G38" s="5" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>CPRX</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>profit</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="n">
+        <v>28.03</v>
+      </c>
+      <c r="D39" s="5" t="n">
+        <v>31.14</v>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>$21</t>
+        </is>
+      </c>
+      <c r="F39" s="21" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="G39" s="5" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>ATHERENERG</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>profit</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="n">
+        <v>960.4</v>
+      </c>
+      <c r="D40" s="5" t="n">
+        <v>979.5</v>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>₹134</t>
+        </is>
+      </c>
+      <c r="F40" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="G40" s="5" t="n">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>LRCX</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>scratch</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="n">
+        <v>346.09</v>
+      </c>
+      <c r="D41" s="5" t="n">
+        <v>346</v>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>$-0</t>
+        </is>
+      </c>
+      <c r="F41" s="23" t="n">
+        <v>-0.03</v>
+      </c>
+      <c r="G41" s="5" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
           <t>DATAPATTNS</t>
         </is>
       </c>
-      <c r="B28" s="5" t="inlineStr">
+      <c r="B42" s="5" t="inlineStr">
         <is>
           <t>loss</t>
         </is>
       </c>
-      <c r="C28" s="5" t="n">
+      <c r="C42" s="5" t="n">
         <v>4805</v>
       </c>
-      <c r="D28" s="5" t="n">
+      <c r="D42" s="5" t="n">
         <v>4400</v>
       </c>
-      <c r="E28" s="5" t="inlineStr">
+      <c r="E42" s="5" t="inlineStr">
         <is>
           <t>₹-4,050</t>
         </is>
       </c>
-      <c r="F28" s="23" t="n">
+      <c r="F42" s="23" t="n">
         <v>-8.4</v>
       </c>
-      <c r="G28" s="5" t="n"/>
+      <c r="G42" s="5" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="27">
+    <mergeCell ref="A7:I7"/>
     <mergeCell ref="D11:I11"/>
+    <mergeCell ref="D27:I27"/>
+    <mergeCell ref="D13:I13"/>
+    <mergeCell ref="D17:I17"/>
+    <mergeCell ref="D16:I16"/>
+    <mergeCell ref="A33:I33"/>
+    <mergeCell ref="D28:I28"/>
+    <mergeCell ref="D18:I18"/>
+    <mergeCell ref="D9:I9"/>
+    <mergeCell ref="D12:I12"/>
+    <mergeCell ref="A4:I4"/>
+    <mergeCell ref="D30:I30"/>
+    <mergeCell ref="D25:I25"/>
+    <mergeCell ref="D15:I15"/>
+    <mergeCell ref="D24:I24"/>
+    <mergeCell ref="D14:I14"/>
+    <mergeCell ref="D29:I29"/>
+    <mergeCell ref="D23:I23"/>
+    <mergeCell ref="D20:I20"/>
+    <mergeCell ref="D26:I26"/>
+    <mergeCell ref="D19:I19"/>
     <mergeCell ref="D10:I10"/>
-    <mergeCell ref="D13:I13"/>
-    <mergeCell ref="A5:I5"/>
-    <mergeCell ref="D14:I14"/>
-    <mergeCell ref="D18:I18"/>
+    <mergeCell ref="D22:I22"/>
+    <mergeCell ref="D31:I31"/>
     <mergeCell ref="A1:I1"/>
-    <mergeCell ref="D17:I17"/>
-    <mergeCell ref="A8:I8"/>
-    <mergeCell ref="D12:I12"/>
-    <mergeCell ref="D16:I16"/>
-    <mergeCell ref="A20:I20"/>
-    <mergeCell ref="D15:I15"/>
+    <mergeCell ref="D21:I21"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4429,7 +4579,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L19"/>
+  <dimension ref="A1:L20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -4518,7 +4668,7 @@
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>SNDK</t>
+          <t>LPG</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
@@ -4528,27 +4678,27 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>profit</t>
+          <t>loss</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="F3" s="5" t="n">
-        <v>0.331205</v>
+        <v>7</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>903.13</v>
+        <v>49.381</v>
       </c>
       <c r="H3" s="13" t="n">
-        <v>1250.83</v>
+        <v>48.21</v>
       </c>
       <c r="I3" s="13" t="n"/>
       <c r="J3" s="13">
@@ -4567,12 +4717,12 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>BSE.NS</t>
+          <t>SNDK</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>INR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
@@ -4582,22 +4732,22 @@
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="F4" s="5" t="n">
-        <v>8</v>
+        <v>0.331205</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>3415.5</v>
+        <v>903.13</v>
       </c>
       <c r="H4" s="13" t="n">
-        <v>3994.53</v>
+        <v>1250.83</v>
       </c>
       <c r="I4" s="13" t="n"/>
       <c r="J4" s="13">
@@ -4616,7 +4766,7 @@
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>KRN</t>
+          <t>BSE.NS</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
@@ -4626,27 +4776,27 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>loss</t>
+          <t>profit</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="F5" s="5" t="n">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>1310</v>
+        <v>3415.5</v>
       </c>
       <c r="H5" s="13" t="n">
-        <v>1197.27</v>
+        <v>3994.53</v>
       </c>
       <c r="I5" s="13" t="n"/>
       <c r="J5" s="13">
@@ -4665,37 +4815,37 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>CPRX</t>
+          <t>KRN</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>INR</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>profit</t>
+          <t>loss</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="F6" s="5" t="n">
-        <v>7.178445</v>
+        <v>22</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>28.03</v>
+        <v>1310</v>
       </c>
       <c r="H6" s="13" t="n">
-        <v>31.14</v>
+        <v>1197.27</v>
       </c>
       <c r="I6" s="13" t="n"/>
       <c r="J6" s="13">
@@ -4714,12 +4864,12 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>ATHERENERG</t>
+          <t>CPRX</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>INR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -4729,22 +4879,22 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="F7" s="5" t="n">
-        <v>7</v>
+        <v>7.178445</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>960.4</v>
+        <v>28.03</v>
       </c>
       <c r="H7" s="13" t="n">
-        <v>979.5</v>
+        <v>31.14</v>
       </c>
       <c r="I7" s="13" t="n"/>
       <c r="J7" s="13">
@@ -4763,37 +4913,37 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>LRCX</t>
+          <t>ATHERENERG</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>INR</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>scratch</t>
+          <t>profit</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="F8" s="5" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>346.09</v>
+        <v>960.4</v>
       </c>
       <c r="H8" s="13" t="n">
-        <v>346</v>
+        <v>979.5</v>
       </c>
       <c r="I8" s="13" t="n"/>
       <c r="J8" s="13">
@@ -4812,37 +4962,37 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>DATAPATTNS</t>
+          <t>LRCX</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>INR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>loss</t>
+          <t>scratch</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="F9" s="5" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>4805</v>
+        <v>346.09</v>
       </c>
       <c r="H9" s="13" t="n">
-        <v>4400</v>
+        <v>346</v>
       </c>
       <c r="I9" s="13" t="n"/>
       <c r="J9" s="13">
@@ -4859,25 +5009,51 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="n"/>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="5" t="n"/>
-      <c r="D10" s="5" t="n"/>
-      <c r="E10" s="5" t="n"/>
-      <c r="F10" s="5" t="n"/>
-      <c r="G10" s="5" t="n"/>
-      <c r="H10" s="5" t="n"/>
-      <c r="I10" s="5" t="n"/>
-      <c r="J10" s="5">
-        <f>IF(F10="","",(H10-G10)*F10)</f>
-        <v/>
-      </c>
-      <c r="K10" s="5">
-        <f>IF(G10="","",(H10-G10)/G10)</f>
-        <v/>
-      </c>
-      <c r="L10" s="5">
-        <f>IF(OR(I10="",G10-I10=0),"",(H10-G10)/(G10-I10))</f>
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>DATAPATTNS</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>loss</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="G10" s="13" t="n">
+        <v>4805</v>
+      </c>
+      <c r="H10" s="13" t="n">
+        <v>4400</v>
+      </c>
+      <c r="I10" s="13" t="n"/>
+      <c r="J10" s="13">
+        <f>(H10-G10)*F10</f>
+        <v/>
+      </c>
+      <c r="K10" s="25">
+        <f>IF(G10&gt;0,(H10-G10)/G10,0)</f>
+        <v/>
+      </c>
+      <c r="L10" s="14">
+        <f>IF(AND(ISNUMBER(I10),G10-I10&lt;&gt;0),(H10-G10)/(G10-I10),"")</f>
         <v/>
       </c>
     </row>
@@ -5085,6 +5261,29 @@
       </c>
       <c r="L19" s="5">
         <f>IF(OR(I19="",G19-I19=0),"",(H19-G19)/(G19-I19))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="n"/>
+      <c r="B20" s="5" t="n"/>
+      <c r="C20" s="5" t="n"/>
+      <c r="D20" s="5" t="n"/>
+      <c r="E20" s="5" t="n"/>
+      <c r="F20" s="5" t="n"/>
+      <c r="G20" s="5" t="n"/>
+      <c r="H20" s="5" t="n"/>
+      <c r="I20" s="5" t="n"/>
+      <c r="J20" s="5">
+        <f>IF(F20="","",(H20-G20)*F20)</f>
+        <v/>
+      </c>
+      <c r="K20" s="5">
+        <f>IF(G20="","",(H20-G20)/G20)</f>
+        <v/>
+      </c>
+      <c r="L20" s="5">
+        <f>IF(OR(I20="",G20-I20=0),"",(H20-G20)/(G20-I20))</f>
         <v/>
       </c>
     </row>
@@ -5473,7 +5672,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J27"/>
+  <dimension ref="A1:J26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5700,7 +5899,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Source: Colgate-Palmolive sale proceeds  |  Pool: ₹1,200,000  |  Risk/trade: 1%  |  Deployed: ₹85,933  |  Cash remaining: ₹1,114,067</t>
+          <t>Source: Colgate-Palmolive sale proceeds  |  Pool: ₹1,200,000  |  Risk/trade: 1%  |  Deployed: ₹32,088  |  Cash remaining: ₹1,165,217</t>
         </is>
       </c>
     </row>
@@ -5816,95 +6015,110 @@
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t>DATAPATTNS</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="n">
-        <v>11</v>
-      </c>
-      <c r="C19" s="13" t="n">
-        <v>4895</v>
-      </c>
-      <c r="D19" s="13" t="n">
-        <v>4895</v>
-      </c>
-      <c r="E19" s="13" t="n">
-        <v>4700</v>
-      </c>
-      <c r="F19" s="13" t="n">
-        <v>4955.9</v>
-      </c>
-      <c r="G19" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="H19" s="6" t="n">
-        <v>2145</v>
-      </c>
-      <c r="I19" s="5" t="inlineStr">
-        <is>
-          <t>override</t>
-        </is>
-      </c>
-      <c r="J19" s="5" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-    </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">↳ History: 2026-08-19/20: Spiked to 'Buy Zone' tag at 4,894.85, vol badge later clarified as a WEEKLY (not single-day) comparison — weaker confirmation than first read. Gave back most of the spike next session (pulled back to ~4785-4790). 2026-08-20: First order (trigger 4,830, R1 pivot reclaim) revised UP to trigger 4,895 / limit 4,950 — now requires reclaiming the actual Buy Zone session price, not just a minor pivot. Better confirmation, still below the 4,955.90 ATH/Core gate. Pilot-sized (11sh, matches the original 25% tranche) — risk to the 4,700 stop is 0.18-0.23% of sleeve regardless of exact fill price. Stop level unchanged at 4,700 (technical support, not adjusted for entry price).
-</t>
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Planned Trades (redeployment of sale proceeds)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>↳ Notes: Reverse-pyramid / 25-50-25 plan. Pilot filled + protected same session — correct discipline, matches the NETWEB lesson. Core (23sh) still gated on close above 4,955.90 ATH on volume + Nifty 50 21D EMA reclaim.</t>
+          <t>None yet — ~₹50L expected free after GILLETTE + COLPAL exits. Plan before redeploying.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>Planned Trades (redeployment of sale proceeds)</t>
+          <t>Closed Swing/Growth Journal</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>None yet — ~₹50L expected free after GILLETTE + COLPAL exits. Plan before redeploying.</t>
-        </is>
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Avg Entry</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>Avg Exit</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>P&amp;L %</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr"/>
+      <c r="I24" s="4" t="inlineStr"/>
+      <c r="J24" s="4" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>DATAPATTNS</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>loss</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="n">
+        <v>4895</v>
+      </c>
+      <c r="D25" s="5" t="n">
+        <v>4650</v>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>₹-2,695</t>
+        </is>
+      </c>
+      <c r="F25" s="23" t="n">
+        <v>-5.01</v>
+      </c>
+      <c r="G25" s="19" t="n">
+        <v>-1</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="inlineStr">
-        <is>
-          <t>Closed Swing/Growth Journal</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>No closed swing/growth trades yet.</t>
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>↳ Stopped out at the GTD SL limit price (4,650) — confirmed by user, exact date pending contract note (placeholder '2026-08-2?'). Loss ₹2,695 (-5.01%), landed right at the planned stop distance — clean execution, stop was placed and protected in the same session as entry. Second consecutive loss on this stock (first was June, -8.4%) — same pattern both times: elite RS/chart quality undermined by a real fundamental crack (June: fresh earnings miss; this time: same Q1FY27 miss plus POOR group rank and Medium conviction). Worth treating any future DATAPATTNS setup with extra skepticism regardless of how clean the chart looks.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="11">
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A23:J23"/>
     <mergeCell ref="A14:J14"/>
     <mergeCell ref="A17:J17"/>
     <mergeCell ref="A18:J18"/>
-    <mergeCell ref="A21:J21"/>
     <mergeCell ref="B8:J8"/>
     <mergeCell ref="A20:J20"/>
     <mergeCell ref="B4:J4"/>

</xml_diff>

<commit_message>
Correct LPG/DATAPATTNS exit dates — order-placement date, not execution
The 'Trade Date' field on the LPG stop-order confirmation screenshot was
the date the GTD stop order was PLACED (Aug 19), not when it executed —
misread as an execution date last time. User confirmed actual exits:
DATAPATTNS "yesterday", LPG "today" (relative to this correction).

Both exit dates set to TBD pending exact calendar confirmation rather
than guessing again. P&L, fill prices, and post-mortem analysis
unchanged — only the date attribution was wrong.

https://claude.ai/code/session_01HhF36NsLiVFyxhhXe4S24m
</commit_message>
<xml_diff>
--- a/examples/swing_monitor/Portfolio_Tracker.xlsx
+++ b/examples/swing_monitor/Portfolio_Tracker.xlsx
@@ -575,7 +575,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-26 16:42  |  USD/INR 95.0  |  prices: override file (2026-08-12T10:29:00+00:00), yfinance off</t>
+          <t>Generated 2026-08-26 16:46  |  USD/INR 95.0  |  prices: override file (2026-08-12T10:29:00+00:00), yfinance off</t>
         </is>
       </c>
     </row>
@@ -4334,9 +4334,7 @@
       <c r="F35" s="23" t="n">
         <v>-2.37</v>
       </c>
-      <c r="G35" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="G35" s="5" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
@@ -4688,7 +4686,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>TBD — confirm today's date</t>
         </is>
       </c>
       <c r="F3" s="5" t="n">
@@ -6108,7 +6106,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>↳ Stopped out at the GTD SL limit price (4,650) — confirmed by user, exact date pending contract note (placeholder '2026-08-2?'). Loss ₹2,695 (-5.01%), landed right at the planned stop distance — clean execution, stop was placed and protected in the same session as entry. Second consecutive loss on this stock (first was June, -8.4%) — same pattern both times: elite RS/chart quality undermined by a real fundamental crack (June: fresh earnings miss; this time: same Q1FY27 miss plus POOR group rank and Medium conviction). Worth treating any future DATAPATTNS setup with extra skepticism regardless of how clean the chart looks.</t>
+          <t>↳ Stopped out at the GTD SL limit price (4,650) — confirmed by user. Exact date pending confirmation. Loss ₹2,695 (-5.01%), landed right at the planned stop distance — clean execution, stop was placed and protected in the same session as entry. Second consecutive loss on this stock (first was June, -8.4%) — same pattern both times: elite RS/chart quality undermined by a real fundamental crack (June: fresh earnings miss; this time: same Q1FY27 miss plus POOR group rank and Medium conviction). Worth treating any future DATAPATTNS setup with extra skepticism regardless of how clean the chart looks.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Finalize LPG and DATAPATTNS exit dates (today confirmed as 2026-08-26)
LPG: exited 2026-08-26, held 7 days (entered 19 Aug). Not a same-day
whipsaw as first assumed — the 7-day hold means the stop-out reflects
several days of price action, not an instant reversal.

DATAPATTNS: exited 2026-08-25 ("yesterday"), held 5 days (entered 20
Aug). hold_days now populated correctly in both journals.

https://claude.ai/code/session_01HhF36NsLiVFyxhhXe4S24m
</commit_message>
<xml_diff>
--- a/examples/swing_monitor/Portfolio_Tracker.xlsx
+++ b/examples/swing_monitor/Portfolio_Tracker.xlsx
@@ -575,7 +575,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-26 16:46  |  USD/INR 95.0  |  prices: override file (2026-08-12T10:29:00+00:00), yfinance off</t>
+          <t>Generated 2026-08-26 16:48  |  USD/INR 95.0  |  prices: override file (2026-08-12T10:29:00+00:00), yfinance off</t>
         </is>
       </c>
     </row>
@@ -4334,7 +4334,9 @@
       <c r="F35" s="23" t="n">
         <v>-2.37</v>
       </c>
-      <c r="G35" s="5" t="n"/>
+      <c r="G35" s="5" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
@@ -4686,7 +4688,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>TBD — confirm today's date</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="F3" s="5" t="n">
@@ -6106,7 +6108,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>↳ Stopped out at the GTD SL limit price (4,650) — confirmed by user. Exact date pending confirmation. Loss ₹2,695 (-5.01%), landed right at the planned stop distance — clean execution, stop was placed and protected in the same session as entry. Second consecutive loss on this stock (first was June, -8.4%) — same pattern both times: elite RS/chart quality undermined by a real fundamental crack (June: fresh earnings miss; this time: same Q1FY27 miss plus POOR group rank and Medium conviction). Worth treating any future DATAPATTNS setup with extra skepticism regardless of how clean the chart looks.</t>
+          <t>↳ Held 5 days (entered 20 Aug, stopped out 25 Aug) at the GTD SL limit price (4,650). Loss ₹2,695 (-5.01%), landed right at the planned stop distance — clean execution, stop was placed and protected in the same session as entry. Second consecutive loss on this stock (first was June, -8.4%) — same pattern both times: elite RS/chart quality undermined by a real fundamental crack (June: fresh earnings miss; this time: same Q1FY27 miss plus POOR group rank and Medium conviction). Worth treating any future DATAPATTNS setup with extra skepticism regardless of how clean the chart looks.</t>
         </is>
       </c>
     </row>

</xml_diff>